<commit_message>
test(appium): run appium tests and update test report
</commit_message>
<xml_diff>
--- a/testing/appium-tests/Test_Report.xlsx
+++ b/testing/appium-tests/Test_Report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2482" uniqueCount="1144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2482" uniqueCount="1146">
   <si>
     <t>GROWMARK MOBILE APP - AUTOMATED TESTING REPORT</t>
   </si>
@@ -1391,7 +1391,7 @@
     <t>TestCase_Sales_15: Submit random sales variation 15</t>
   </si>
   <si>
-    <t>Item: "Item 1", Quantity: 110, Date: Today</t>
+    <t>Item: "Item 1", Quantity: 84, Date: Today</t>
   </si>
   <si>
     <t>Sales record saved and threshold check triggered</t>
@@ -1406,7 +1406,7 @@
     <t>TestCase_Sales_16: Submit random sales variation 16</t>
   </si>
   <si>
-    <t>Item: "Item 2", Quantity: 26, Date: Today</t>
+    <t>Item: "Item 2", Quantity: 97, Date: Today</t>
   </si>
   <si>
     <t>TC111</t>
@@ -1415,7 +1415,7 @@
     <t>TestCase_Sales_17: Submit random sales variation 17</t>
   </si>
   <si>
-    <t>Item: "Item 3", Quantity: 58, Date: Today</t>
+    <t>Item: "Item 3", Quantity: 124, Date: Today</t>
   </si>
   <si>
     <t>TC112</t>
@@ -1424,7 +1424,7 @@
     <t>TestCase_Sales_18: Submit random sales variation 18</t>
   </si>
   <si>
-    <t>Item: "Item 4", Quantity: 198, Date: Today</t>
+    <t>Item: "Item 4", Quantity: 139, Date: Today</t>
   </si>
   <si>
     <t>TC113</t>
@@ -1433,7 +1433,7 @@
     <t>TestCase_Sales_19: Submit random sales variation 19</t>
   </si>
   <si>
-    <t>Item: "Item 5", Quantity: 185, Date: Today</t>
+    <t>Item: "Item 5", Quantity: 61, Date: Today</t>
   </si>
   <si>
     <t>TC114</t>
@@ -1442,7 +1442,7 @@
     <t>TestCase_Sales_20: Submit random sales variation 20</t>
   </si>
   <si>
-    <t>Item: "Item 1", Quantity: 109, Date: Today</t>
+    <t>Item: "Item 1", Quantity: 192, Date: Today</t>
   </si>
   <si>
     <t>TC115</t>
@@ -1451,7 +1451,7 @@
     <t>TestCase_Sales_21: Submit random sales variation 21</t>
   </si>
   <si>
-    <t>Item: "Item 2", Quantity: 104, Date: Today</t>
+    <t>Item: "Item 2", Quantity: 114, Date: Today</t>
   </si>
   <si>
     <t>TC116</t>
@@ -1460,7 +1460,7 @@
     <t>TestCase_Sales_22: Submit random sales variation 22</t>
   </si>
   <si>
-    <t>Item: "Item 3", Quantity: 85, Date: Today</t>
+    <t>Item: "Item 3", Quantity: 81, Date: Today</t>
   </si>
   <si>
     <t>TC117</t>
@@ -1469,7 +1469,7 @@
     <t>TestCase_Sales_23: Submit random sales variation 23</t>
   </si>
   <si>
-    <t>Item: "Item 4", Quantity: 32, Date: Today</t>
+    <t>Item: "Item 4", Quantity: 75, Date: Today</t>
   </si>
   <si>
     <t>TC118</t>
@@ -1478,7 +1478,7 @@
     <t>TestCase_Sales_24: Submit random sales variation 24</t>
   </si>
   <si>
-    <t>Item: "Item 5", Quantity: 69, Date: Today</t>
+    <t>Item: "Item 5", Quantity: 54, Date: Today</t>
   </si>
   <si>
     <t>TC119</t>
@@ -1487,7 +1487,7 @@
     <t>TestCase_Sales_25: Submit random sales variation 25</t>
   </si>
   <si>
-    <t>Item: "Item 1", Quantity: 146, Date: Today</t>
+    <t>Item: "Item 1", Quantity: 135, Date: Today</t>
   </si>
   <si>
     <t>TC120</t>
@@ -1496,7 +1496,7 @@
     <t>TestCase_Sales_26: Submit random sales variation 26</t>
   </si>
   <si>
-    <t>Item: "Item 2", Quantity: 72, Date: Today</t>
+    <t>Item: "Item 2", Quantity: 62, Date: Today</t>
   </si>
   <si>
     <t>TC121</t>
@@ -1505,7 +1505,7 @@
     <t>TestCase_Sales_27: Submit random sales variation 27</t>
   </si>
   <si>
-    <t>Item: "Item 3", Quantity: 177, Date: Today</t>
+    <t>Item: "Item 3", Quantity: 80, Date: Today</t>
   </si>
   <si>
     <t>TC122</t>
@@ -1514,7 +1514,7 @@
     <t>TestCase_Sales_28: Submit random sales variation 28</t>
   </si>
   <si>
-    <t>Item: "Item 4", Quantity: 55, Date: Today</t>
+    <t>Item: "Item 4", Quantity: 179, Date: Today</t>
   </si>
   <si>
     <t>TC123</t>
@@ -1523,7 +1523,7 @@
     <t>TestCase_Sales_29: Submit random sales variation 29</t>
   </si>
   <si>
-    <t>Item: "Item 5", Quantity: 26, Date: Today</t>
+    <t>Item: "Item 5", Quantity: 58, Date: Today</t>
   </si>
   <si>
     <t>TC124</t>
@@ -1532,7 +1532,7 @@
     <t>TestCase_Sales_30: Submit random sales variation 30</t>
   </si>
   <si>
-    <t>Item: "Item 1", Quantity: 79, Date: Today</t>
+    <t>Item: "Item 1", Quantity: 95, Date: Today</t>
   </si>
   <si>
     <t>TC125</t>
@@ -1541,7 +1541,7 @@
     <t>TestCase_Sales_31: Submit random sales variation 31</t>
   </si>
   <si>
-    <t>Item: "Item 2", Quantity: 52, Date: Today</t>
+    <t>Item: "Item 2", Quantity: 85, Date: Today</t>
   </si>
   <si>
     <t>TC126</t>
@@ -1550,7 +1550,7 @@
     <t>TestCase_Sales_32: Submit random sales variation 32</t>
   </si>
   <si>
-    <t>Item: "Item 3", Quantity: 26, Date: Today</t>
+    <t>Item: "Item 3", Quantity: 190, Date: Today</t>
   </si>
   <si>
     <t>TC127</t>
@@ -1559,7 +1559,7 @@
     <t>TestCase_Sales_33: Submit random sales variation 33</t>
   </si>
   <si>
-    <t>Item: "Item 4", Quantity: 5, Date: Today</t>
+    <t>Item: "Item 4", Quantity: 14, Date: Today</t>
   </si>
   <si>
     <t>TC128</t>
@@ -1568,7 +1568,7 @@
     <t>TestCase_Sales_34: Submit random sales variation 34</t>
   </si>
   <si>
-    <t>Item: "Item 5", Quantity: 189, Date: Today</t>
+    <t>Item: "Item 5", Quantity: 72, Date: Today</t>
   </si>
   <si>
     <t>TC129</t>
@@ -1577,7 +1577,7 @@
     <t>TestCase_Sales_35: Submit random sales variation 35</t>
   </si>
   <si>
-    <t>Item: "Item 1", Quantity: 45, Date: Today</t>
+    <t>Item: "Item 1", Quantity: 44, Date: Today</t>
   </si>
   <si>
     <t>TC130</t>
@@ -1586,7 +1586,7 @@
     <t>TestCase_Sales_36: Submit random sales variation 36</t>
   </si>
   <si>
-    <t>Item: "Item 2", Quantity: 168, Date: Today</t>
+    <t>Item: "Item 2", Quantity: 149, Date: Today</t>
   </si>
   <si>
     <t>TC131</t>
@@ -1595,7 +1595,7 @@
     <t>TestCase_Sales_37: Submit random sales variation 37</t>
   </si>
   <si>
-    <t>Item: "Item 3", Quantity: 78, Date: Today</t>
+    <t>Item: "Item 3", Quantity: 158, Date: Today</t>
   </si>
   <si>
     <t>TC132</t>
@@ -1604,7 +1604,7 @@
     <t>TestCase_Sales_38: Submit random sales variation 38</t>
   </si>
   <si>
-    <t>Item: "Item 4", Quantity: 101, Date: Today</t>
+    <t>Item: "Item 4", Quantity: 107, Date: Today</t>
   </si>
   <si>
     <t>TC133</t>
@@ -1613,7 +1613,7 @@
     <t>TestCase_Sales_39: Submit random sales variation 39</t>
   </si>
   <si>
-    <t>Item: "Item 5", Quantity: 165, Date: Today</t>
+    <t>Item: "Item 5", Quantity: 179, Date: Today</t>
   </si>
   <si>
     <t>TC134</t>
@@ -1622,7 +1622,7 @@
     <t>TestCase_Sales_40: Submit random sales variation 40</t>
   </si>
   <si>
-    <t>Item: "Item 1", Quantity: 153, Date: Today</t>
+    <t>Item: "Item 1", Quantity: 155, Date: Today</t>
   </si>
   <si>
     <t>TC135</t>
@@ -1631,7 +1631,7 @@
     <t>TestCase_Sales_41: Submit random sales variation 41</t>
   </si>
   <si>
-    <t>Item: "Item 2", Quantity: 79, Date: Today</t>
+    <t>Item: "Item 2", Quantity: 172, Date: Today</t>
   </si>
   <si>
     <t>TC136</t>
@@ -1640,7 +1640,7 @@
     <t>TestCase_Sales_42: Submit random sales variation 42</t>
   </si>
   <si>
-    <t>Item: "Item 3", Quantity: 8, Date: Today</t>
+    <t>Item: "Item 3", Quantity: 189, Date: Today</t>
   </si>
   <si>
     <t>TC137</t>
@@ -1649,7 +1649,7 @@
     <t>TestCase_Sales_43: Submit random sales variation 43</t>
   </si>
   <si>
-    <t>Item: "Item 4", Quantity: 19, Date: Today</t>
+    <t>Item: "Item 4", Quantity: 191, Date: Today</t>
   </si>
   <si>
     <t>TC138</t>
@@ -1658,7 +1658,7 @@
     <t>TestCase_Sales_44: Submit random sales variation 44</t>
   </si>
   <si>
-    <t>Item: "Item 5", Quantity: 144, Date: Today</t>
+    <t>Item: "Item 5", Quantity: 114, Date: Today</t>
   </si>
   <si>
     <t>TC139</t>
@@ -1667,7 +1667,7 @@
     <t>TestCase_Sales_45: Submit random sales variation 45</t>
   </si>
   <si>
-    <t>Item: "Item 1", Quantity: 171, Date: Today</t>
+    <t>Item: "Item 1", Quantity: 136, Date: Today</t>
   </si>
   <si>
     <t>TC140</t>
@@ -1676,7 +1676,7 @@
     <t>TestCase_Sales_46: Submit random sales variation 46</t>
   </si>
   <si>
-    <t>Item: "Item 2", Quantity: 37, Date: Today</t>
+    <t>Item: "Item 2", Quantity: 87, Date: Today</t>
   </si>
   <si>
     <t>TC141</t>
@@ -1685,7 +1685,7 @@
     <t>TestCase_Sales_47: Submit random sales variation 47</t>
   </si>
   <si>
-    <t>Item: "Item 3", Quantity: 107, Date: Today</t>
+    <t>Item: "Item 3", Quantity: 110, Date: Today</t>
   </si>
   <si>
     <t>TC142</t>
@@ -1694,7 +1694,7 @@
     <t>TestCase_Sales_48: Submit random sales variation 48</t>
   </si>
   <si>
-    <t>Item: "Item 4", Quantity: 40, Date: Today</t>
+    <t>Item: "Item 4", Quantity: 86, Date: Today</t>
   </si>
   <si>
     <t>TC143</t>
@@ -1703,7 +1703,7 @@
     <t>TestCase_Sales_49: Submit random sales variation 49</t>
   </si>
   <si>
-    <t>Item: "Item 5", Quantity: 45, Date: Today</t>
+    <t>Item: "Item 5", Quantity: 68, Date: Today</t>
   </si>
   <si>
     <t>TC144</t>
@@ -1712,7 +1712,7 @@
     <t>TestCase_Sales_50: Submit random sales variation 50</t>
   </si>
   <si>
-    <t>Item: "Item 1", Quantity: 70, Date: Today</t>
+    <t>Item: "Item 1", Quantity: 194, Date: Today</t>
   </si>
   <si>
     <t>TC145</t>
@@ -2876,10 +2876,10 @@
     <t>TC251</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_09: Score 35 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 35</t>
+    <t>TestCase_HealthScore_09: Score 29 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 29</t>
   </si>
   <si>
     <t>Verdict: "Immediate Action Needed" displayed</t>
@@ -2891,133 +2891,139 @@
     <t>TC252</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_10: Score 9 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 9</t>
+    <t>TestCase_HealthScore_10: Score 98 shows "Thriving" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 98</t>
+  </si>
+  <si>
+    <t>Verdict: "Thriving" displayed</t>
   </si>
   <si>
     <t>TC253</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_11: Score 13 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 13</t>
+    <t>TestCase_HealthScore_11: Score 33 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 33</t>
   </si>
   <si>
     <t>TC254</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_12: Score 0 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 0</t>
+    <t>TestCase_HealthScore_12: Score 25 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 25</t>
   </si>
   <si>
     <t>TC255</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_13: Score 85 shows "Thriving" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 85</t>
-  </si>
-  <si>
-    <t>Verdict: "Thriving" displayed</t>
+    <t>TestCase_HealthScore_13: Score 16 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 16</t>
   </si>
   <si>
     <t>TC256</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_14: Score 36 shows "Immediate Action Needed" verdict</t>
+    <t>TestCase_HealthScore_14: Score 43 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 43</t>
+  </si>
+  <si>
+    <t>TC257</t>
+  </si>
+  <si>
+    <t>TestCase_HealthScore_15: Score 44 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 44</t>
+  </si>
+  <si>
+    <t>TC258</t>
+  </si>
+  <si>
+    <t>TestCase_HealthScore_16: Score 77 shows "Work in Progress" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 77</t>
+  </si>
+  <si>
+    <t>Verdict: "Work in Progress" displayed</t>
+  </si>
+  <si>
+    <t>TC259</t>
+  </si>
+  <si>
+    <t>TestCase_HealthScore_17: Score 59 shows "Work in Progress" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 59</t>
+  </si>
+  <si>
+    <t>TC260</t>
+  </si>
+  <si>
+    <t>TestCase_HealthScore_18: Score 18 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 18</t>
+  </si>
+  <si>
+    <t>TC261</t>
+  </si>
+  <si>
+    <t>TestCase_HealthScore_19: Score 36 shows "Immediate Action Needed" verdict</t>
   </si>
   <si>
     <t>Simulated score: 36</t>
   </si>
   <si>
-    <t>TC257</t>
-  </si>
-  <si>
-    <t>TestCase_HealthScore_15: Score 0 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>TC258</t>
-  </si>
-  <si>
-    <t>TestCase_HealthScore_16: Score 94 shows "Thriving" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 94</t>
-  </si>
-  <si>
-    <t>TC259</t>
-  </si>
-  <si>
-    <t>TestCase_HealthScore_17: Score 68 shows "Work in Progress" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 68</t>
-  </si>
-  <si>
-    <t>Verdict: "Work in Progress" displayed</t>
-  </si>
-  <si>
-    <t>TC260</t>
-  </si>
-  <si>
-    <t>TestCase_HealthScore_18: Score 60 shows "Work in Progress" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 60</t>
-  </si>
-  <si>
-    <t>TC261</t>
-  </si>
-  <si>
-    <t>TestCase_HealthScore_19: Score 68 shows "Work in Progress" verdict</t>
-  </si>
-  <si>
     <t>TC262</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_20: Score 94 shows "Thriving" verdict</t>
+    <t>TestCase_HealthScore_20: Score 45 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 45</t>
   </si>
   <si>
     <t>TC263</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_21: Score 57 shows "Work in Progress" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 57</t>
+    <t>TestCase_HealthScore_21: Score 59 shows "Work in Progress" verdict</t>
   </si>
   <si>
     <t>TC264</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_22: Score 4 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 4</t>
+    <t>TestCase_HealthScore_22: Score 38 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 38</t>
   </si>
   <si>
     <t>TC265</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_23: Score 69 shows "Work in Progress" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 69</t>
+    <t>TestCase_HealthScore_23: Score 11 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 11</t>
   </si>
   <si>
     <t>TC266</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_24: Score 46 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 46</t>
+    <t>TestCase_HealthScore_24: Score 53 shows "Work in Progress" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 53</t>
   </si>
   <si>
     <t>TC267</t>
@@ -4499,7 +4505,7 @@
         <v>9</v>
       </c>
       <c r="H2" s="11">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="I2" s="11" t="s">
         <v>1</v>
@@ -4528,7 +4534,7 @@
         <v>9</v>
       </c>
       <c r="H3" s="13">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="I3" s="13" t="s">
         <v>1</v>
@@ -4557,7 +4563,7 @@
         <v>9</v>
       </c>
       <c r="H4" s="11">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I4" s="11" t="s">
         <v>1</v>
@@ -4586,7 +4592,7 @@
         <v>9</v>
       </c>
       <c r="H5" s="13">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="I5" s="13" t="s">
         <v>1</v>
@@ -4615,7 +4621,7 @@
         <v>9</v>
       </c>
       <c r="H6" s="11">
-        <v>88</v>
+        <v>31</v>
       </c>
       <c r="I6" s="11" t="s">
         <v>1</v>
@@ -4644,7 +4650,7 @@
         <v>9</v>
       </c>
       <c r="H7" s="13">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="I7" s="13" t="s">
         <v>1</v>
@@ -4673,7 +4679,7 @@
         <v>9</v>
       </c>
       <c r="H8" s="11">
-        <v>16</v>
+        <v>76</v>
       </c>
       <c r="I8" s="11" t="s">
         <v>1</v>
@@ -4702,7 +4708,7 @@
         <v>9</v>
       </c>
       <c r="H9" s="13">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="I9" s="13" t="s">
         <v>1</v>
@@ -4731,7 +4737,7 @@
         <v>9</v>
       </c>
       <c r="H10" s="11">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="I10" s="11" t="s">
         <v>1</v>
@@ -4760,7 +4766,7 @@
         <v>9</v>
       </c>
       <c r="H11" s="13">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I11" s="13" t="s">
         <v>1</v>
@@ -4789,7 +4795,7 @@
         <v>9</v>
       </c>
       <c r="H12" s="11">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="I12" s="11" t="s">
         <v>1</v>
@@ -4818,7 +4824,7 @@
         <v>9</v>
       </c>
       <c r="H13" s="13">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="I13" s="13" t="s">
         <v>1</v>
@@ -4847,7 +4853,7 @@
         <v>9</v>
       </c>
       <c r="H14" s="11">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="I14" s="11" t="s">
         <v>1</v>
@@ -4876,7 +4882,7 @@
         <v>9</v>
       </c>
       <c r="H15" s="13">
-        <v>58</v>
+        <v>80</v>
       </c>
       <c r="I15" s="13" t="s">
         <v>1</v>
@@ -4905,7 +4911,7 @@
         <v>9</v>
       </c>
       <c r="H16" s="11">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="I16" s="11" t="s">
         <v>1</v>
@@ -4934,7 +4940,7 @@
         <v>9</v>
       </c>
       <c r="H17" s="13">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="I17" s="13" t="s">
         <v>1</v>
@@ -4963,7 +4969,7 @@
         <v>9</v>
       </c>
       <c r="H18" s="11">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="I18" s="11" t="s">
         <v>1</v>
@@ -4992,7 +4998,7 @@
         <v>9</v>
       </c>
       <c r="H19" s="13">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="I19" s="13" t="s">
         <v>1</v>
@@ -5021,7 +5027,7 @@
         <v>9</v>
       </c>
       <c r="H20" s="11">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I20" s="11" t="s">
         <v>1</v>
@@ -5050,7 +5056,7 @@
         <v>9</v>
       </c>
       <c r="H21" s="13">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I21" s="13" t="s">
         <v>1</v>
@@ -5079,7 +5085,7 @@
         <v>9</v>
       </c>
       <c r="H22" s="11">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="I22" s="11" t="s">
         <v>1</v>
@@ -5108,7 +5114,7 @@
         <v>9</v>
       </c>
       <c r="H23" s="13">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="I23" s="13" t="s">
         <v>1</v>
@@ -5137,7 +5143,7 @@
         <v>9</v>
       </c>
       <c r="H24" s="11">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="I24" s="11" t="s">
         <v>1</v>
@@ -5166,7 +5172,7 @@
         <v>9</v>
       </c>
       <c r="H25" s="13">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="I25" s="13" t="s">
         <v>1</v>
@@ -5195,7 +5201,7 @@
         <v>9</v>
       </c>
       <c r="H26" s="11">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="I26" s="11" t="s">
         <v>1</v>
@@ -5224,7 +5230,7 @@
         <v>9</v>
       </c>
       <c r="H27" s="13">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="I27" s="13" t="s">
         <v>1</v>
@@ -5253,7 +5259,7 @@
         <v>9</v>
       </c>
       <c r="H28" s="11">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="I28" s="11" t="s">
         <v>1</v>
@@ -5282,7 +5288,7 @@
         <v>9</v>
       </c>
       <c r="H29" s="13">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="I29" s="13" t="s">
         <v>1</v>
@@ -5311,7 +5317,7 @@
         <v>9</v>
       </c>
       <c r="H30" s="11">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="I30" s="11" t="s">
         <v>1</v>
@@ -5340,7 +5346,7 @@
         <v>9</v>
       </c>
       <c r="H31" s="13">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="I31" s="13" t="s">
         <v>1</v>
@@ -5369,7 +5375,7 @@
         <v>9</v>
       </c>
       <c r="H32" s="11">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="I32" s="11" t="s">
         <v>1</v>
@@ -5398,7 +5404,7 @@
         <v>9</v>
       </c>
       <c r="H33" s="13">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I33" s="13" t="s">
         <v>1</v>
@@ -5427,7 +5433,7 @@
         <v>9</v>
       </c>
       <c r="H34" s="11">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="I34" s="11" t="s">
         <v>1</v>
@@ -5456,7 +5462,7 @@
         <v>9</v>
       </c>
       <c r="H35" s="13">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="I35" s="13" t="s">
         <v>1</v>
@@ -5485,7 +5491,7 @@
         <v>9</v>
       </c>
       <c r="H36" s="11">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="I36" s="11" t="s">
         <v>1</v>
@@ -5514,7 +5520,7 @@
         <v>9</v>
       </c>
       <c r="H37" s="13">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="I37" s="13" t="s">
         <v>1</v>
@@ -5543,7 +5549,7 @@
         <v>9</v>
       </c>
       <c r="H38" s="11">
-        <v>34</v>
+        <v>81</v>
       </c>
       <c r="I38" s="11" t="s">
         <v>1</v>
@@ -5572,7 +5578,7 @@
         <v>9</v>
       </c>
       <c r="H39" s="13">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="I39" s="13" t="s">
         <v>1</v>
@@ -5601,7 +5607,7 @@
         <v>9</v>
       </c>
       <c r="H40" s="11">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="I40" s="11" t="s">
         <v>1</v>
@@ -5630,7 +5636,7 @@
         <v>9</v>
       </c>
       <c r="H41" s="13">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="I41" s="13" t="s">
         <v>1</v>
@@ -5659,7 +5665,7 @@
         <v>9</v>
       </c>
       <c r="H42" s="11">
-        <v>13</v>
+        <v>82</v>
       </c>
       <c r="I42" s="11" t="s">
         <v>1</v>
@@ -5688,7 +5694,7 @@
         <v>9</v>
       </c>
       <c r="H43" s="13">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="I43" s="13" t="s">
         <v>1</v>
@@ -5717,7 +5723,7 @@
         <v>9</v>
       </c>
       <c r="H44" s="11">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="I44" s="11" t="s">
         <v>1</v>
@@ -5746,7 +5752,7 @@
         <v>9</v>
       </c>
       <c r="H45" s="13">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="I45" s="13" t="s">
         <v>1</v>
@@ -5775,7 +5781,7 @@
         <v>9</v>
       </c>
       <c r="H46" s="11">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="I46" s="11" t="s">
         <v>1</v>
@@ -5804,7 +5810,7 @@
         <v>9</v>
       </c>
       <c r="H47" s="13">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="I47" s="13" t="s">
         <v>1</v>
@@ -5833,7 +5839,7 @@
         <v>9</v>
       </c>
       <c r="H48" s="11">
-        <v>29</v>
+        <v>82</v>
       </c>
       <c r="I48" s="11" t="s">
         <v>1</v>
@@ -5862,7 +5868,7 @@
         <v>9</v>
       </c>
       <c r="H49" s="13">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="I49" s="13" t="s">
         <v>1</v>
@@ -5891,7 +5897,7 @@
         <v>9</v>
       </c>
       <c r="H50" s="11">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="I50" s="11" t="s">
         <v>1</v>
@@ -5920,7 +5926,7 @@
         <v>9</v>
       </c>
       <c r="H51" s="13">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I51" s="13" t="s">
         <v>1</v>
@@ -5949,7 +5955,7 @@
         <v>9</v>
       </c>
       <c r="H52" s="11">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="I52" s="11" t="s">
         <v>1</v>
@@ -5978,7 +5984,7 @@
         <v>9</v>
       </c>
       <c r="H53" s="13">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="I53" s="13" t="s">
         <v>1</v>
@@ -6007,7 +6013,7 @@
         <v>9</v>
       </c>
       <c r="H54" s="11">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="I54" s="11" t="s">
         <v>1</v>
@@ -6036,7 +6042,7 @@
         <v>9</v>
       </c>
       <c r="H55" s="13">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="I55" s="13" t="s">
         <v>1</v>
@@ -6065,7 +6071,7 @@
         <v>9</v>
       </c>
       <c r="H56" s="11">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="I56" s="11" t="s">
         <v>1</v>
@@ -6094,7 +6100,7 @@
         <v>9</v>
       </c>
       <c r="H57" s="13">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="I57" s="13" t="s">
         <v>1</v>
@@ -6123,7 +6129,7 @@
         <v>9</v>
       </c>
       <c r="H58" s="11">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="I58" s="11" t="s">
         <v>1</v>
@@ -6152,7 +6158,7 @@
         <v>9</v>
       </c>
       <c r="H59" s="13">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="I59" s="13" t="s">
         <v>1</v>
@@ -6181,7 +6187,7 @@
         <v>9</v>
       </c>
       <c r="H60" s="11">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="I60" s="11" t="s">
         <v>1</v>
@@ -6210,7 +6216,7 @@
         <v>9</v>
       </c>
       <c r="H61" s="13">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="I61" s="13" t="s">
         <v>1</v>
@@ -6239,7 +6245,7 @@
         <v>9</v>
       </c>
       <c r="H62" s="11">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="I62" s="11" t="s">
         <v>1</v>
@@ -6268,7 +6274,7 @@
         <v>9</v>
       </c>
       <c r="H63" s="13">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="I63" s="13" t="s">
         <v>1</v>
@@ -6326,7 +6332,7 @@
         <v>9</v>
       </c>
       <c r="H65" s="13">
-        <v>69</v>
+        <v>10</v>
       </c>
       <c r="I65" s="13" t="s">
         <v>1</v>
@@ -6355,7 +6361,7 @@
         <v>9</v>
       </c>
       <c r="H66" s="11">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="I66" s="11" t="s">
         <v>1</v>
@@ -6384,7 +6390,7 @@
         <v>9</v>
       </c>
       <c r="H67" s="13">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="I67" s="13" t="s">
         <v>1</v>
@@ -6413,7 +6419,7 @@
         <v>9</v>
       </c>
       <c r="H68" s="11">
-        <v>31</v>
+        <v>64</v>
       </c>
       <c r="I68" s="11" t="s">
         <v>1</v>
@@ -6442,7 +6448,7 @@
         <v>9</v>
       </c>
       <c r="H69" s="13">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="I69" s="13" t="s">
         <v>1</v>
@@ -6471,7 +6477,7 @@
         <v>9</v>
       </c>
       <c r="H70" s="11">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="I70" s="11" t="s">
         <v>1</v>
@@ -6500,7 +6506,7 @@
         <v>9</v>
       </c>
       <c r="H71" s="13">
-        <v>81</v>
+        <v>29</v>
       </c>
       <c r="I71" s="13" t="s">
         <v>1</v>
@@ -6529,7 +6535,7 @@
         <v>9</v>
       </c>
       <c r="H72" s="11">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="I72" s="11" t="s">
         <v>1</v>
@@ -6558,7 +6564,7 @@
         <v>9</v>
       </c>
       <c r="H73" s="13">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="I73" s="13" t="s">
         <v>1</v>
@@ -6587,7 +6593,7 @@
         <v>9</v>
       </c>
       <c r="H74" s="11">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="I74" s="11" t="s">
         <v>1</v>
@@ -6616,7 +6622,7 @@
         <v>9</v>
       </c>
       <c r="H75" s="13">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="I75" s="13" t="s">
         <v>1</v>
@@ -6645,7 +6651,7 @@
         <v>9</v>
       </c>
       <c r="H76" s="11">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="I76" s="11" t="s">
         <v>1</v>
@@ -6674,7 +6680,7 @@
         <v>9</v>
       </c>
       <c r="H77" s="13">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="I77" s="13" t="s">
         <v>1</v>
@@ -6703,7 +6709,7 @@
         <v>9</v>
       </c>
       <c r="H78" s="11">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I78" s="11" t="s">
         <v>1</v>
@@ -6732,7 +6738,7 @@
         <v>9</v>
       </c>
       <c r="H79" s="13">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="I79" s="13" t="s">
         <v>1</v>
@@ -6761,7 +6767,7 @@
         <v>9</v>
       </c>
       <c r="H80" s="11">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="I80" s="11" t="s">
         <v>1</v>
@@ -6790,7 +6796,7 @@
         <v>9</v>
       </c>
       <c r="H81" s="13">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="I81" s="13" t="s">
         <v>1</v>
@@ -6819,7 +6825,7 @@
         <v>9</v>
       </c>
       <c r="H82" s="11">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I82" s="11" t="s">
         <v>1</v>
@@ -6848,7 +6854,7 @@
         <v>9</v>
       </c>
       <c r="H83" s="13">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="I83" s="13" t="s">
         <v>1</v>
@@ -6877,7 +6883,7 @@
         <v>9</v>
       </c>
       <c r="H84" s="11">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="I84" s="11" t="s">
         <v>1</v>
@@ -6906,7 +6912,7 @@
         <v>9</v>
       </c>
       <c r="H85" s="13">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="I85" s="13" t="s">
         <v>1</v>
@@ -6935,7 +6941,7 @@
         <v>9</v>
       </c>
       <c r="H86" s="11">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="I86" s="11" t="s">
         <v>1</v>
@@ -6964,7 +6970,7 @@
         <v>9</v>
       </c>
       <c r="H87" s="13">
-        <v>81</v>
+        <v>10</v>
       </c>
       <c r="I87" s="13" t="s">
         <v>1</v>
@@ -6993,7 +6999,7 @@
         <v>9</v>
       </c>
       <c r="H88" s="11">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="I88" s="11" t="s">
         <v>1</v>
@@ -7022,7 +7028,7 @@
         <v>9</v>
       </c>
       <c r="H89" s="13">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="I89" s="13" t="s">
         <v>1</v>
@@ -7051,7 +7057,7 @@
         <v>9</v>
       </c>
       <c r="H90" s="11">
-        <v>87</v>
+        <v>26</v>
       </c>
       <c r="I90" s="11" t="s">
         <v>1</v>
@@ -7080,7 +7086,7 @@
         <v>9</v>
       </c>
       <c r="H91" s="13">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="I91" s="13" t="s">
         <v>1</v>
@@ -7109,7 +7115,7 @@
         <v>9</v>
       </c>
       <c r="H92" s="11">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="I92" s="11" t="s">
         <v>1</v>
@@ -7138,7 +7144,7 @@
         <v>9</v>
       </c>
       <c r="H93" s="13">
-        <v>29</v>
+        <v>73</v>
       </c>
       <c r="I93" s="13" t="s">
         <v>1</v>
@@ -7167,7 +7173,7 @@
         <v>9</v>
       </c>
       <c r="H94" s="11">
-        <v>24</v>
+        <v>68</v>
       </c>
       <c r="I94" s="11" t="s">
         <v>1</v>
@@ -7196,7 +7202,7 @@
         <v>9</v>
       </c>
       <c r="H95" s="13">
-        <v>16</v>
+        <v>83</v>
       </c>
       <c r="I95" s="13" t="s">
         <v>1</v>
@@ -7225,7 +7231,7 @@
         <v>9</v>
       </c>
       <c r="H96" s="11">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="I96" s="11" t="s">
         <v>1</v>
@@ -7254,7 +7260,7 @@
         <v>9</v>
       </c>
       <c r="H97" s="13">
-        <v>47</v>
+        <v>87</v>
       </c>
       <c r="I97" s="13" t="s">
         <v>1</v>
@@ -7283,7 +7289,7 @@
         <v>9</v>
       </c>
       <c r="H98" s="11">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="I98" s="11" t="s">
         <v>1</v>
@@ -7312,7 +7318,7 @@
         <v>9</v>
       </c>
       <c r="H99" s="13">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I99" s="13" t="s">
         <v>1</v>
@@ -7341,7 +7347,7 @@
         <v>9</v>
       </c>
       <c r="H100" s="11">
-        <v>81</v>
+        <v>37</v>
       </c>
       <c r="I100" s="11" t="s">
         <v>1</v>
@@ -7370,7 +7376,7 @@
         <v>9</v>
       </c>
       <c r="H101" s="13">
-        <v>62</v>
+        <v>10</v>
       </c>
       <c r="I101" s="13" t="s">
         <v>1</v>
@@ -7399,7 +7405,7 @@
         <v>9</v>
       </c>
       <c r="H102" s="11">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="I102" s="11" t="s">
         <v>1</v>
@@ -7428,7 +7434,7 @@
         <v>9</v>
       </c>
       <c r="H103" s="13">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="I103" s="13" t="s">
         <v>1</v>
@@ -7457,7 +7463,7 @@
         <v>9</v>
       </c>
       <c r="H104" s="11">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="I104" s="11" t="s">
         <v>1</v>
@@ -7486,7 +7492,7 @@
         <v>9</v>
       </c>
       <c r="H105" s="13">
-        <v>17</v>
+        <v>76</v>
       </c>
       <c r="I105" s="13" t="s">
         <v>1</v>
@@ -7515,7 +7521,7 @@
         <v>9</v>
       </c>
       <c r="H106" s="11">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="I106" s="11" t="s">
         <v>1</v>
@@ -7544,7 +7550,7 @@
         <v>9</v>
       </c>
       <c r="H107" s="13">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I107" s="13" t="s">
         <v>1</v>
@@ -7573,7 +7579,7 @@
         <v>9</v>
       </c>
       <c r="H108" s="11">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="I108" s="11" t="s">
         <v>1</v>
@@ -7602,7 +7608,7 @@
         <v>9</v>
       </c>
       <c r="H109" s="13">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="I109" s="13" t="s">
         <v>1</v>
@@ -7631,7 +7637,7 @@
         <v>9</v>
       </c>
       <c r="H110" s="11">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="I110" s="11" t="s">
         <v>1</v>
@@ -7660,7 +7666,7 @@
         <v>9</v>
       </c>
       <c r="H111" s="13">
-        <v>31</v>
+        <v>84</v>
       </c>
       <c r="I111" s="13" t="s">
         <v>1</v>
@@ -7689,7 +7695,7 @@
         <v>9</v>
       </c>
       <c r="H112" s="11">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="I112" s="11" t="s">
         <v>1</v>
@@ -7718,7 +7724,7 @@
         <v>9</v>
       </c>
       <c r="H113" s="13">
-        <v>80</v>
+        <v>48</v>
       </c>
       <c r="I113" s="13" t="s">
         <v>1</v>
@@ -7747,7 +7753,7 @@
         <v>9</v>
       </c>
       <c r="H114" s="11">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I114" s="11" t="s">
         <v>1</v>
@@ -7776,7 +7782,7 @@
         <v>9</v>
       </c>
       <c r="H115" s="13">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="I115" s="13" t="s">
         <v>1</v>
@@ -7805,7 +7811,7 @@
         <v>9</v>
       </c>
       <c r="H116" s="11">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="I116" s="11" t="s">
         <v>1</v>
@@ -7834,7 +7840,7 @@
         <v>9</v>
       </c>
       <c r="H117" s="13">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="I117" s="13" t="s">
         <v>1</v>
@@ -7863,7 +7869,7 @@
         <v>9</v>
       </c>
       <c r="H118" s="11">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="I118" s="11" t="s">
         <v>1</v>
@@ -7892,7 +7898,7 @@
         <v>9</v>
       </c>
       <c r="H119" s="13">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="I119" s="13" t="s">
         <v>1</v>
@@ -7921,7 +7927,7 @@
         <v>9</v>
       </c>
       <c r="H120" s="11">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="I120" s="11" t="s">
         <v>1</v>
@@ -7950,7 +7956,7 @@
         <v>9</v>
       </c>
       <c r="H121" s="13">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="I121" s="13" t="s">
         <v>1</v>
@@ -7979,7 +7985,7 @@
         <v>9</v>
       </c>
       <c r="H122" s="11">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="I122" s="11" t="s">
         <v>1</v>
@@ -8008,7 +8014,7 @@
         <v>9</v>
       </c>
       <c r="H123" s="13">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="I123" s="13" t="s">
         <v>1</v>
@@ -8037,7 +8043,7 @@
         <v>9</v>
       </c>
       <c r="H124" s="11">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="I124" s="11" t="s">
         <v>1</v>
@@ -8066,7 +8072,7 @@
         <v>9</v>
       </c>
       <c r="H125" s="13">
-        <v>69</v>
+        <v>26</v>
       </c>
       <c r="I125" s="13" t="s">
         <v>1</v>
@@ -8095,7 +8101,7 @@
         <v>9</v>
       </c>
       <c r="H126" s="11">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="I126" s="11" t="s">
         <v>1</v>
@@ -8124,7 +8130,7 @@
         <v>9</v>
       </c>
       <c r="H127" s="13">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="I127" s="13" t="s">
         <v>1</v>
@@ -8153,7 +8159,7 @@
         <v>9</v>
       </c>
       <c r="H128" s="11">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="I128" s="11" t="s">
         <v>1</v>
@@ -8182,7 +8188,7 @@
         <v>9</v>
       </c>
       <c r="H129" s="13">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="I129" s="13" t="s">
         <v>1</v>
@@ -8211,7 +8217,7 @@
         <v>9</v>
       </c>
       <c r="H130" s="11">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="I130" s="11" t="s">
         <v>1</v>
@@ -8240,7 +8246,7 @@
         <v>9</v>
       </c>
       <c r="H131" s="13">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="I131" s="13" t="s">
         <v>1</v>
@@ -8269,7 +8275,7 @@
         <v>9</v>
       </c>
       <c r="H132" s="11">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="I132" s="11" t="s">
         <v>1</v>
@@ -8298,7 +8304,7 @@
         <v>9</v>
       </c>
       <c r="H133" s="13">
-        <v>85</v>
+        <v>29</v>
       </c>
       <c r="I133" s="13" t="s">
         <v>1</v>
@@ -8327,7 +8333,7 @@
         <v>9</v>
       </c>
       <c r="H134" s="11">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="I134" s="11" t="s">
         <v>1</v>
@@ -8356,7 +8362,7 @@
         <v>9</v>
       </c>
       <c r="H135" s="13">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="I135" s="13" t="s">
         <v>1</v>
@@ -8385,7 +8391,7 @@
         <v>9</v>
       </c>
       <c r="H136" s="11">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I136" s="11" t="s">
         <v>1</v>
@@ -8414,7 +8420,7 @@
         <v>9</v>
       </c>
       <c r="H137" s="13">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="I137" s="13" t="s">
         <v>1</v>
@@ -8443,7 +8449,7 @@
         <v>9</v>
       </c>
       <c r="H138" s="11">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="I138" s="11" t="s">
         <v>1</v>
@@ -8472,7 +8478,7 @@
         <v>9</v>
       </c>
       <c r="H139" s="13">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="I139" s="13" t="s">
         <v>1</v>
@@ -8501,7 +8507,7 @@
         <v>9</v>
       </c>
       <c r="H140" s="11">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="I140" s="11" t="s">
         <v>1</v>
@@ -8530,7 +8536,7 @@
         <v>9</v>
       </c>
       <c r="H141" s="13">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="I141" s="13" t="s">
         <v>1</v>
@@ -8559,7 +8565,7 @@
         <v>9</v>
       </c>
       <c r="H142" s="11">
-        <v>67</v>
+        <v>43</v>
       </c>
       <c r="I142" s="11" t="s">
         <v>1</v>
@@ -8588,7 +8594,7 @@
         <v>9</v>
       </c>
       <c r="H143" s="13">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="I143" s="13" t="s">
         <v>1</v>
@@ -8617,7 +8623,7 @@
         <v>9</v>
       </c>
       <c r="H144" s="11">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I144" s="11" t="s">
         <v>1</v>
@@ -8646,7 +8652,7 @@
         <v>9</v>
       </c>
       <c r="H145" s="13">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="I145" s="13" t="s">
         <v>1</v>
@@ -8704,7 +8710,7 @@
         <v>9</v>
       </c>
       <c r="H147" s="13">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="I147" s="13" t="s">
         <v>1</v>
@@ -8733,7 +8739,7 @@
         <v>9</v>
       </c>
       <c r="H148" s="11">
-        <v>86</v>
+        <v>32</v>
       </c>
       <c r="I148" s="11" t="s">
         <v>1</v>
@@ -8762,7 +8768,7 @@
         <v>9</v>
       </c>
       <c r="H149" s="13">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="I149" s="13" t="s">
         <v>1</v>
@@ -8791,7 +8797,7 @@
         <v>9</v>
       </c>
       <c r="H150" s="11">
-        <v>26</v>
+        <v>79</v>
       </c>
       <c r="I150" s="11" t="s">
         <v>1</v>
@@ -8820,7 +8826,7 @@
         <v>9</v>
       </c>
       <c r="H151" s="13">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="I151" s="13" t="s">
         <v>1</v>
@@ -8849,7 +8855,7 @@
         <v>9</v>
       </c>
       <c r="H152" s="11">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="I152" s="11" t="s">
         <v>1</v>
@@ -8878,7 +8884,7 @@
         <v>9</v>
       </c>
       <c r="H153" s="13">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="I153" s="13" t="s">
         <v>1</v>
@@ -8907,7 +8913,7 @@
         <v>9</v>
       </c>
       <c r="H154" s="11">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="I154" s="11" t="s">
         <v>1</v>
@@ -8936,7 +8942,7 @@
         <v>9</v>
       </c>
       <c r="H155" s="13">
-        <v>30</v>
+        <v>84</v>
       </c>
       <c r="I155" s="13" t="s">
         <v>1</v>
@@ -8965,7 +8971,7 @@
         <v>9</v>
       </c>
       <c r="H156" s="11">
-        <v>84</v>
+        <v>25</v>
       </c>
       <c r="I156" s="11" t="s">
         <v>1</v>
@@ -8994,7 +9000,7 @@
         <v>9</v>
       </c>
       <c r="H157" s="13">
-        <v>83</v>
+        <v>47</v>
       </c>
       <c r="I157" s="13" t="s">
         <v>1</v>
@@ -9023,7 +9029,7 @@
         <v>9</v>
       </c>
       <c r="H158" s="11">
-        <v>13</v>
+        <v>80</v>
       </c>
       <c r="I158" s="11" t="s">
         <v>1</v>
@@ -9052,7 +9058,7 @@
         <v>9</v>
       </c>
       <c r="H159" s="13">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="I159" s="13" t="s">
         <v>1</v>
@@ -9081,7 +9087,7 @@
         <v>9</v>
       </c>
       <c r="H160" s="11">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="I160" s="11" t="s">
         <v>1</v>
@@ -9110,7 +9116,7 @@
         <v>9</v>
       </c>
       <c r="H161" s="13">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I161" s="13" t="s">
         <v>1</v>
@@ -9139,7 +9145,7 @@
         <v>9</v>
       </c>
       <c r="H162" s="11">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="I162" s="11" t="s">
         <v>1</v>
@@ -9168,7 +9174,7 @@
         <v>9</v>
       </c>
       <c r="H163" s="13">
-        <v>81</v>
+        <v>18</v>
       </c>
       <c r="I163" s="13" t="s">
         <v>1</v>
@@ -9197,7 +9203,7 @@
         <v>9</v>
       </c>
       <c r="H164" s="11">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="I164" s="11" t="s">
         <v>1</v>
@@ -9226,7 +9232,7 @@
         <v>9</v>
       </c>
       <c r="H165" s="13">
-        <v>42</v>
+        <v>75</v>
       </c>
       <c r="I165" s="13" t="s">
         <v>1</v>
@@ -9255,7 +9261,7 @@
         <v>9</v>
       </c>
       <c r="H166" s="11">
-        <v>52</v>
+        <v>87</v>
       </c>
       <c r="I166" s="11" t="s">
         <v>1</v>
@@ -9284,7 +9290,7 @@
         <v>9</v>
       </c>
       <c r="H167" s="13">
-        <v>35</v>
+        <v>77</v>
       </c>
       <c r="I167" s="13" t="s">
         <v>1</v>
@@ -9313,7 +9319,7 @@
         <v>9</v>
       </c>
       <c r="H168" s="11">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="I168" s="11" t="s">
         <v>1</v>
@@ -9342,7 +9348,7 @@
         <v>9</v>
       </c>
       <c r="H169" s="13">
-        <v>42</v>
+        <v>82</v>
       </c>
       <c r="I169" s="13" t="s">
         <v>1</v>
@@ -9371,7 +9377,7 @@
         <v>9</v>
       </c>
       <c r="H170" s="11">
-        <v>63</v>
+        <v>23</v>
       </c>
       <c r="I170" s="11" t="s">
         <v>1</v>
@@ -9400,7 +9406,7 @@
         <v>9</v>
       </c>
       <c r="H171" s="13">
-        <v>79</v>
+        <v>13</v>
       </c>
       <c r="I171" s="13" t="s">
         <v>1</v>
@@ -9429,7 +9435,7 @@
         <v>9</v>
       </c>
       <c r="H172" s="11">
-        <v>73</v>
+        <v>29</v>
       </c>
       <c r="I172" s="11" t="s">
         <v>1</v>
@@ -9458,7 +9464,7 @@
         <v>9</v>
       </c>
       <c r="H173" s="13">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="I173" s="13" t="s">
         <v>1</v>
@@ -9487,7 +9493,7 @@
         <v>9</v>
       </c>
       <c r="H174" s="11">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="I174" s="11" t="s">
         <v>1</v>
@@ -9516,7 +9522,7 @@
         <v>9</v>
       </c>
       <c r="H175" s="13">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="I175" s="13" t="s">
         <v>1</v>
@@ -9545,7 +9551,7 @@
         <v>9</v>
       </c>
       <c r="H176" s="11">
-        <v>87</v>
+        <v>13</v>
       </c>
       <c r="I176" s="11" t="s">
         <v>1</v>
@@ -9574,7 +9580,7 @@
         <v>9</v>
       </c>
       <c r="H177" s="13">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="I177" s="13" t="s">
         <v>1</v>
@@ -9603,7 +9609,7 @@
         <v>9</v>
       </c>
       <c r="H178" s="11">
-        <v>88</v>
+        <v>36</v>
       </c>
       <c r="I178" s="11" t="s">
         <v>1</v>
@@ -9632,7 +9638,7 @@
         <v>9</v>
       </c>
       <c r="H179" s="13">
-        <v>70</v>
+        <v>33</v>
       </c>
       <c r="I179" s="13" t="s">
         <v>1</v>
@@ -9661,7 +9667,7 @@
         <v>9</v>
       </c>
       <c r="H180" s="11">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="I180" s="11" t="s">
         <v>1</v>
@@ -9690,7 +9696,7 @@
         <v>9</v>
       </c>
       <c r="H181" s="13">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="I181" s="13" t="s">
         <v>1</v>
@@ -9719,7 +9725,7 @@
         <v>9</v>
       </c>
       <c r="H182" s="11">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="I182" s="11" t="s">
         <v>1</v>
@@ -9748,7 +9754,7 @@
         <v>9</v>
       </c>
       <c r="H183" s="13">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="I183" s="13" t="s">
         <v>1</v>
@@ -9777,7 +9783,7 @@
         <v>9</v>
       </c>
       <c r="H184" s="11">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="I184" s="11" t="s">
         <v>1</v>
@@ -9806,7 +9812,7 @@
         <v>9</v>
       </c>
       <c r="H185" s="13">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="I185" s="13" t="s">
         <v>1</v>
@@ -9835,7 +9841,7 @@
         <v>9</v>
       </c>
       <c r="H186" s="11">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="I186" s="11" t="s">
         <v>1</v>
@@ -9864,7 +9870,7 @@
         <v>9</v>
       </c>
       <c r="H187" s="13">
-        <v>27</v>
+        <v>57</v>
       </c>
       <c r="I187" s="13" t="s">
         <v>1</v>
@@ -9893,7 +9899,7 @@
         <v>9</v>
       </c>
       <c r="H188" s="11">
-        <v>22</v>
+        <v>87</v>
       </c>
       <c r="I188" s="11" t="s">
         <v>1</v>
@@ -9922,7 +9928,7 @@
         <v>9</v>
       </c>
       <c r="H189" s="13">
-        <v>13</v>
+        <v>77</v>
       </c>
       <c r="I189" s="13" t="s">
         <v>1</v>
@@ -9951,7 +9957,7 @@
         <v>9</v>
       </c>
       <c r="H190" s="11">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="I190" s="11" t="s">
         <v>1</v>
@@ -9980,7 +9986,7 @@
         <v>9</v>
       </c>
       <c r="H191" s="13">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="I191" s="13" t="s">
         <v>1</v>
@@ -10009,7 +10015,7 @@
         <v>9</v>
       </c>
       <c r="H192" s="11">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="I192" s="11" t="s">
         <v>1</v>
@@ -10038,7 +10044,7 @@
         <v>9</v>
       </c>
       <c r="H193" s="13">
-        <v>41</v>
+        <v>84</v>
       </c>
       <c r="I193" s="13" t="s">
         <v>1</v>
@@ -10067,7 +10073,7 @@
         <v>9</v>
       </c>
       <c r="H194" s="11">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="I194" s="11" t="s">
         <v>1</v>
@@ -10096,7 +10102,7 @@
         <v>9</v>
       </c>
       <c r="H195" s="13">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="I195" s="13" t="s">
         <v>1</v>
@@ -10125,7 +10131,7 @@
         <v>9</v>
       </c>
       <c r="H196" s="11">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="I196" s="11" t="s">
         <v>1</v>
@@ -10154,7 +10160,7 @@
         <v>9</v>
       </c>
       <c r="H197" s="13">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="I197" s="13" t="s">
         <v>1</v>
@@ -10183,7 +10189,7 @@
         <v>9</v>
       </c>
       <c r="H198" s="11">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="I198" s="11" t="s">
         <v>1</v>
@@ -10212,7 +10218,7 @@
         <v>9</v>
       </c>
       <c r="H199" s="13">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="I199" s="13" t="s">
         <v>1</v>
@@ -10241,7 +10247,7 @@
         <v>9</v>
       </c>
       <c r="H200" s="11">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I200" s="11" t="s">
         <v>1</v>
@@ -10270,7 +10276,7 @@
         <v>9</v>
       </c>
       <c r="H201" s="13">
-        <v>65</v>
+        <v>37</v>
       </c>
       <c r="I201" s="13" t="s">
         <v>1</v>
@@ -10299,7 +10305,7 @@
         <v>9</v>
       </c>
       <c r="H202" s="11">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="I202" s="11" t="s">
         <v>1</v>
@@ -10328,7 +10334,7 @@
         <v>9</v>
       </c>
       <c r="H203" s="13">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="I203" s="13" t="s">
         <v>1</v>
@@ -10357,7 +10363,7 @@
         <v>9</v>
       </c>
       <c r="H204" s="11">
-        <v>79</v>
+        <v>23</v>
       </c>
       <c r="I204" s="11" t="s">
         <v>1</v>
@@ -10386,7 +10392,7 @@
         <v>9</v>
       </c>
       <c r="H205" s="13">
-        <v>89</v>
+        <v>32</v>
       </c>
       <c r="I205" s="13" t="s">
         <v>1</v>
@@ -10415,7 +10421,7 @@
         <v>9</v>
       </c>
       <c r="H206" s="11">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="I206" s="11" t="s">
         <v>1</v>
@@ -10444,7 +10450,7 @@
         <v>9</v>
       </c>
       <c r="H207" s="13">
-        <v>87</v>
+        <v>41</v>
       </c>
       <c r="I207" s="13" t="s">
         <v>1</v>
@@ -10473,7 +10479,7 @@
         <v>9</v>
       </c>
       <c r="H208" s="11">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I208" s="11" t="s">
         <v>1</v>
@@ -10502,7 +10508,7 @@
         <v>9</v>
       </c>
       <c r="H209" s="13">
-        <v>24</v>
+        <v>89</v>
       </c>
       <c r="I209" s="13" t="s">
         <v>1</v>
@@ -10531,7 +10537,7 @@
         <v>9</v>
       </c>
       <c r="H210" s="11">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="I210" s="11" t="s">
         <v>1</v>
@@ -10560,7 +10566,7 @@
         <v>9</v>
       </c>
       <c r="H211" s="13">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="I211" s="13" t="s">
         <v>1</v>
@@ -10589,7 +10595,7 @@
         <v>9</v>
       </c>
       <c r="H212" s="11">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="I212" s="11" t="s">
         <v>1</v>
@@ -10618,7 +10624,7 @@
         <v>9</v>
       </c>
       <c r="H213" s="13">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="I213" s="13" t="s">
         <v>1</v>
@@ -10647,7 +10653,7 @@
         <v>9</v>
       </c>
       <c r="H214" s="11">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="I214" s="11" t="s">
         <v>1</v>
@@ -10676,7 +10682,7 @@
         <v>9</v>
       </c>
       <c r="H215" s="13">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="I215" s="13" t="s">
         <v>1</v>
@@ -10705,7 +10711,7 @@
         <v>9</v>
       </c>
       <c r="H216" s="11">
-        <v>27</v>
+        <v>89</v>
       </c>
       <c r="I216" s="11" t="s">
         <v>1</v>
@@ -10734,7 +10740,7 @@
         <v>9</v>
       </c>
       <c r="H217" s="13">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I217" s="13" t="s">
         <v>1</v>
@@ -10763,7 +10769,7 @@
         <v>9</v>
       </c>
       <c r="H218" s="11">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="I218" s="11" t="s">
         <v>1</v>
@@ -10792,7 +10798,7 @@
         <v>9</v>
       </c>
       <c r="H219" s="13">
-        <v>82</v>
+        <v>52</v>
       </c>
       <c r="I219" s="13" t="s">
         <v>1</v>
@@ -10821,7 +10827,7 @@
         <v>9</v>
       </c>
       <c r="H220" s="11">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="I220" s="11" t="s">
         <v>1</v>
@@ -10850,7 +10856,7 @@
         <v>9</v>
       </c>
       <c r="H221" s="13">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="I221" s="13" t="s">
         <v>1</v>
@@ -10879,7 +10885,7 @@
         <v>9</v>
       </c>
       <c r="H222" s="11">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="I222" s="11" t="s">
         <v>1</v>
@@ -10908,7 +10914,7 @@
         <v>9</v>
       </c>
       <c r="H223" s="13">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="I223" s="13" t="s">
         <v>1</v>
@@ -10937,7 +10943,7 @@
         <v>9</v>
       </c>
       <c r="H224" s="11">
-        <v>15</v>
+        <v>76</v>
       </c>
       <c r="I224" s="11" t="s">
         <v>1</v>
@@ -10966,7 +10972,7 @@
         <v>9</v>
       </c>
       <c r="H225" s="13">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="I225" s="13" t="s">
         <v>1</v>
@@ -10995,7 +11001,7 @@
         <v>9</v>
       </c>
       <c r="H226" s="11">
-        <v>54</v>
+        <v>84</v>
       </c>
       <c r="I226" s="11" t="s">
         <v>1</v>
@@ -11024,7 +11030,7 @@
         <v>9</v>
       </c>
       <c r="H227" s="13">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="I227" s="13" t="s">
         <v>1</v>
@@ -11053,7 +11059,7 @@
         <v>9</v>
       </c>
       <c r="H228" s="11">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I228" s="11" t="s">
         <v>1</v>
@@ -11082,7 +11088,7 @@
         <v>9</v>
       </c>
       <c r="H229" s="13">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="I229" s="13" t="s">
         <v>1</v>
@@ -11111,7 +11117,7 @@
         <v>9</v>
       </c>
       <c r="H230" s="11">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="I230" s="11" t="s">
         <v>1</v>
@@ -11140,7 +11146,7 @@
         <v>9</v>
       </c>
       <c r="H231" s="13">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="I231" s="13" t="s">
         <v>1</v>
@@ -11169,7 +11175,7 @@
         <v>9</v>
       </c>
       <c r="H232" s="11">
-        <v>79</v>
+        <v>35</v>
       </c>
       <c r="I232" s="11" t="s">
         <v>1</v>
@@ -11198,7 +11204,7 @@
         <v>9</v>
       </c>
       <c r="H233" s="13">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="I233" s="13" t="s">
         <v>1</v>
@@ -11227,7 +11233,7 @@
         <v>9</v>
       </c>
       <c r="H234" s="11">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="I234" s="11" t="s">
         <v>1</v>
@@ -11256,7 +11262,7 @@
         <v>9</v>
       </c>
       <c r="H235" s="13">
-        <v>88</v>
+        <v>40</v>
       </c>
       <c r="I235" s="13" t="s">
         <v>1</v>
@@ -11285,7 +11291,7 @@
         <v>9</v>
       </c>
       <c r="H236" s="11">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="I236" s="11" t="s">
         <v>1</v>
@@ -11314,7 +11320,7 @@
         <v>9</v>
       </c>
       <c r="H237" s="13">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I237" s="13" t="s">
         <v>1</v>
@@ -11343,7 +11349,7 @@
         <v>9</v>
       </c>
       <c r="H238" s="11">
-        <v>12</v>
+        <v>86</v>
       </c>
       <c r="I238" s="11" t="s">
         <v>1</v>
@@ -11372,7 +11378,7 @@
         <v>9</v>
       </c>
       <c r="H239" s="13">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="I239" s="13" t="s">
         <v>1</v>
@@ -11401,7 +11407,7 @@
         <v>9</v>
       </c>
       <c r="H240" s="11">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="I240" s="11" t="s">
         <v>1</v>
@@ -11430,7 +11436,7 @@
         <v>9</v>
       </c>
       <c r="H241" s="13">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="I241" s="13" t="s">
         <v>1</v>
@@ -11459,7 +11465,7 @@
         <v>9</v>
       </c>
       <c r="H242" s="11">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="I242" s="11" t="s">
         <v>1</v>
@@ -11488,7 +11494,7 @@
         <v>9</v>
       </c>
       <c r="H243" s="13">
-        <v>17</v>
+        <v>84</v>
       </c>
       <c r="I243" s="13" t="s">
         <v>1</v>
@@ -11517,7 +11523,7 @@
         <v>9</v>
       </c>
       <c r="H244" s="11">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="I244" s="11" t="s">
         <v>1</v>
@@ -11546,7 +11552,7 @@
         <v>9</v>
       </c>
       <c r="H245" s="13">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="I245" s="13" t="s">
         <v>1</v>
@@ -11575,7 +11581,7 @@
         <v>9</v>
       </c>
       <c r="H246" s="11">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="I246" s="11" t="s">
         <v>1</v>
@@ -11604,7 +11610,7 @@
         <v>9</v>
       </c>
       <c r="H247" s="13">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="I247" s="13" t="s">
         <v>1</v>
@@ -11633,7 +11639,7 @@
         <v>9</v>
       </c>
       <c r="H248" s="11">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="I248" s="11" t="s">
         <v>1</v>
@@ -11662,7 +11668,7 @@
         <v>9</v>
       </c>
       <c r="H249" s="13">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="I249" s="13" t="s">
         <v>1</v>
@@ -11691,7 +11697,7 @@
         <v>9</v>
       </c>
       <c r="H250" s="11">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="I250" s="11" t="s">
         <v>1</v>
@@ -11720,7 +11726,7 @@
         <v>9</v>
       </c>
       <c r="H251" s="13">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="I251" s="13" t="s">
         <v>1</v>
@@ -11749,7 +11755,7 @@
         <v>9</v>
       </c>
       <c r="H252" s="11">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="I252" s="11" t="s">
         <v>1</v>
@@ -11769,7 +11775,7 @@
         <v>960</v>
       </c>
       <c r="E253" s="13" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="F253" s="13" t="s">
         <v>957</v>
@@ -11778,7 +11784,7 @@
         <v>9</v>
       </c>
       <c r="H253" s="13">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I253" s="13" t="s">
         <v>1</v>
@@ -11786,16 +11792,16 @@
     </row>
     <row r="254" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A254" s="11" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="B254" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C254" s="11" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="D254" s="11" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="E254" s="11" t="s">
         <v>956</v>
@@ -11807,7 +11813,7 @@
         <v>9</v>
       </c>
       <c r="H254" s="11">
-        <v>36</v>
+        <v>88</v>
       </c>
       <c r="I254" s="11" t="s">
         <v>1</v>
@@ -11815,16 +11821,16 @@
     </row>
     <row r="255" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A255" s="13" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="B255" s="13" t="s">
         <v>24</v>
       </c>
       <c r="C255" s="13" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="D255" s="13" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="E255" s="13" t="s">
         <v>956</v>
@@ -11836,7 +11842,7 @@
         <v>9</v>
       </c>
       <c r="H255" s="13">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I255" s="13" t="s">
         <v>1</v>
@@ -11844,19 +11850,19 @@
     </row>
     <row r="256" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A256" s="11" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="B256" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C256" s="11" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="D256" s="11" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="E256" s="11" t="s">
-        <v>970</v>
+        <v>956</v>
       </c>
       <c r="F256" s="11" t="s">
         <v>957</v>
@@ -11865,7 +11871,7 @@
         <v>9</v>
       </c>
       <c r="H256" s="11">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="I256" s="11" t="s">
         <v>1</v>
@@ -11894,7 +11900,7 @@
         <v>9</v>
       </c>
       <c r="H257" s="13">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="I257" s="13" t="s">
         <v>1</v>
@@ -11911,7 +11917,7 @@
         <v>975</v>
       </c>
       <c r="D258" s="11" t="s">
-        <v>966</v>
+        <v>976</v>
       </c>
       <c r="E258" s="11" t="s">
         <v>956</v>
@@ -11923,7 +11929,7 @@
         <v>9</v>
       </c>
       <c r="H258" s="11">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="I258" s="11" t="s">
         <v>1</v>
@@ -11931,19 +11937,19 @@
     </row>
     <row r="259" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A259" s="13" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="B259" s="13" t="s">
         <v>24</v>
       </c>
       <c r="C259" s="13" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="D259" s="13" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="E259" s="13" t="s">
-        <v>970</v>
+        <v>980</v>
       </c>
       <c r="F259" s="13" t="s">
         <v>957</v>
@@ -11952,7 +11958,7 @@
         <v>9</v>
       </c>
       <c r="H259" s="13">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="I259" s="13" t="s">
         <v>1</v>
@@ -11960,19 +11966,19 @@
     </row>
     <row r="260" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A260" s="11" t="s">
-        <v>979</v>
+        <v>981</v>
       </c>
       <c r="B260" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C260" s="11" t="s">
+        <v>982</v>
+      </c>
+      <c r="D260" s="11" t="s">
+        <v>983</v>
+      </c>
+      <c r="E260" s="11" t="s">
         <v>980</v>
-      </c>
-      <c r="D260" s="11" t="s">
-        <v>981</v>
-      </c>
-      <c r="E260" s="11" t="s">
-        <v>982</v>
       </c>
       <c r="F260" s="11" t="s">
         <v>957</v>
@@ -11981,7 +11987,7 @@
         <v>9</v>
       </c>
       <c r="H260" s="11">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="I260" s="11" t="s">
         <v>1</v>
@@ -11989,19 +11995,19 @@
     </row>
     <row r="261" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A261" s="13" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="B261" s="13" t="s">
         <v>24</v>
       </c>
       <c r="C261" s="13" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="D261" s="13" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="E261" s="13" t="s">
-        <v>982</v>
+        <v>956</v>
       </c>
       <c r="F261" s="13" t="s">
         <v>957</v>
@@ -12010,7 +12016,7 @@
         <v>9</v>
       </c>
       <c r="H261" s="13">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="I261" s="13" t="s">
         <v>1</v>
@@ -12018,19 +12024,19 @@
     </row>
     <row r="262" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A262" s="11" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="B262" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C262" s="11" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="D262" s="11" t="s">
-        <v>981</v>
+        <v>989</v>
       </c>
       <c r="E262" s="11" t="s">
-        <v>982</v>
+        <v>956</v>
       </c>
       <c r="F262" s="11" t="s">
         <v>957</v>
@@ -12039,7 +12045,7 @@
         <v>9</v>
       </c>
       <c r="H262" s="11">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="I262" s="11" t="s">
         <v>1</v>
@@ -12047,19 +12053,19 @@
     </row>
     <row r="263" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A263" s="13" t="s">
-        <v>988</v>
+        <v>990</v>
       </c>
       <c r="B263" s="13" t="s">
         <v>24</v>
       </c>
       <c r="C263" s="13" t="s">
-        <v>989</v>
+        <v>991</v>
       </c>
       <c r="D263" s="13" t="s">
-        <v>978</v>
+        <v>992</v>
       </c>
       <c r="E263" s="13" t="s">
-        <v>970</v>
+        <v>956</v>
       </c>
       <c r="F263" s="13" t="s">
         <v>957</v>
@@ -12068,7 +12074,7 @@
         <v>9</v>
       </c>
       <c r="H263" s="13">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="I263" s="13" t="s">
         <v>1</v>
@@ -12076,19 +12082,19 @@
     </row>
     <row r="264" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A264" s="11" t="s">
-        <v>990</v>
+        <v>993</v>
       </c>
       <c r="B264" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C264" s="11" t="s">
-        <v>991</v>
+        <v>994</v>
       </c>
       <c r="D264" s="11" t="s">
-        <v>992</v>
+        <v>983</v>
       </c>
       <c r="E264" s="11" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
       <c r="F264" s="11" t="s">
         <v>957</v>
@@ -12097,7 +12103,7 @@
         <v>9</v>
       </c>
       <c r="H264" s="11">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="I264" s="11" t="s">
         <v>1</v>
@@ -12105,16 +12111,16 @@
     </row>
     <row r="265" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A265" s="13" t="s">
-        <v>993</v>
+        <v>995</v>
       </c>
       <c r="B265" s="13" t="s">
         <v>24</v>
       </c>
       <c r="C265" s="13" t="s">
-        <v>994</v>
+        <v>996</v>
       </c>
       <c r="D265" s="13" t="s">
-        <v>995</v>
+        <v>997</v>
       </c>
       <c r="E265" s="13" t="s">
         <v>956</v>
@@ -12126,7 +12132,7 @@
         <v>9</v>
       </c>
       <c r="H265" s="13">
-        <v>45</v>
+        <v>87</v>
       </c>
       <c r="I265" s="13" t="s">
         <v>1</v>
@@ -12134,19 +12140,19 @@
     </row>
     <row r="266" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A266" s="11" t="s">
-        <v>996</v>
+        <v>998</v>
       </c>
       <c r="B266" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C266" s="11" t="s">
-        <v>997</v>
+        <v>999</v>
       </c>
       <c r="D266" s="11" t="s">
-        <v>998</v>
+        <v>1000</v>
       </c>
       <c r="E266" s="11" t="s">
-        <v>982</v>
+        <v>956</v>
       </c>
       <c r="F266" s="11" t="s">
         <v>957</v>
@@ -12155,7 +12161,7 @@
         <v>9</v>
       </c>
       <c r="H266" s="11">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="I266" s="11" t="s">
         <v>1</v>
@@ -12163,19 +12169,19 @@
     </row>
     <row r="267" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A267" s="13" t="s">
-        <v>999</v>
+        <v>1001</v>
       </c>
       <c r="B267" s="13" t="s">
         <v>24</v>
       </c>
       <c r="C267" s="13" t="s">
-        <v>1000</v>
+        <v>1002</v>
       </c>
       <c r="D267" s="13" t="s">
-        <v>1001</v>
+        <v>1003</v>
       </c>
       <c r="E267" s="13" t="s">
-        <v>956</v>
+        <v>980</v>
       </c>
       <c r="F267" s="13" t="s">
         <v>957</v>
@@ -12184,7 +12190,7 @@
         <v>9</v>
       </c>
       <c r="H267" s="13">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="I267" s="13" t="s">
         <v>1</v>
@@ -12192,28 +12198,28 @@
     </row>
     <row r="268" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A268" s="11" t="s">
-        <v>1002</v>
+        <v>1004</v>
       </c>
       <c r="B268" s="11" t="s">
         <v>25</v>
       </c>
       <c r="C268" s="11" t="s">
-        <v>1003</v>
+        <v>1005</v>
       </c>
       <c r="D268" s="11" t="s">
-        <v>1004</v>
+        <v>1006</v>
       </c>
       <c r="E268" s="11" t="s">
-        <v>1005</v>
+        <v>1007</v>
       </c>
       <c r="F268" s="11" t="s">
-        <v>1006</v>
+        <v>1008</v>
       </c>
       <c r="G268" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H268" s="11">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="I268" s="11" t="s">
         <v>1</v>
@@ -12221,28 +12227,28 @@
     </row>
     <row r="269" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A269" s="13" t="s">
-        <v>1007</v>
+        <v>1009</v>
       </c>
       <c r="B269" s="13" t="s">
         <v>25</v>
       </c>
       <c r="C269" s="13" t="s">
-        <v>1008</v>
+        <v>1010</v>
       </c>
       <c r="D269" s="13" t="s">
-        <v>1009</v>
+        <v>1011</v>
       </c>
       <c r="E269" s="13" t="s">
-        <v>1010</v>
+        <v>1012</v>
       </c>
       <c r="F269" s="13" t="s">
-        <v>1011</v>
+        <v>1013</v>
       </c>
       <c r="G269" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H269" s="13">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="I269" s="13" t="s">
         <v>1</v>
@@ -12250,28 +12256,28 @@
     </row>
     <row r="270" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A270" s="11" t="s">
-        <v>1012</v>
+        <v>1014</v>
       </c>
       <c r="B270" s="11" t="s">
         <v>25</v>
       </c>
       <c r="C270" s="11" t="s">
-        <v>1013</v>
+        <v>1015</v>
       </c>
       <c r="D270" s="11" t="s">
-        <v>1014</v>
+        <v>1016</v>
       </c>
       <c r="E270" s="11" t="s">
-        <v>1015</v>
+        <v>1017</v>
       </c>
       <c r="F270" s="11" t="s">
-        <v>1016</v>
+        <v>1018</v>
       </c>
       <c r="G270" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H270" s="11">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="I270" s="11" t="s">
         <v>1</v>
@@ -12279,28 +12285,28 @@
     </row>
     <row r="271" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A271" s="13" t="s">
-        <v>1017</v>
+        <v>1019</v>
       </c>
       <c r="B271" s="13" t="s">
         <v>25</v>
       </c>
       <c r="C271" s="13" t="s">
-        <v>1018</v>
+        <v>1020</v>
       </c>
       <c r="D271" s="13" t="s">
-        <v>1019</v>
+        <v>1021</v>
       </c>
       <c r="E271" s="13" t="s">
-        <v>1020</v>
+        <v>1022</v>
       </c>
       <c r="F271" s="13" t="s">
-        <v>1021</v>
+        <v>1023</v>
       </c>
       <c r="G271" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H271" s="13">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="I271" s="13" t="s">
         <v>1</v>
@@ -12308,28 +12314,28 @@
     </row>
     <row r="272" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A272" s="11" t="s">
-        <v>1022</v>
+        <v>1024</v>
       </c>
       <c r="B272" s="11" t="s">
         <v>25</v>
       </c>
       <c r="C272" s="11" t="s">
-        <v>1023</v>
+        <v>1025</v>
       </c>
       <c r="D272" s="11" t="s">
-        <v>1024</v>
+        <v>1026</v>
       </c>
       <c r="E272" s="11" t="s">
-        <v>1025</v>
+        <v>1027</v>
       </c>
       <c r="F272" s="11" t="s">
-        <v>1026</v>
+        <v>1028</v>
       </c>
       <c r="G272" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H272" s="11">
-        <v>37</v>
+        <v>73</v>
       </c>
       <c r="I272" s="11" t="s">
         <v>1</v>
@@ -12337,28 +12343,28 @@
     </row>
     <row r="273" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A273" s="13" t="s">
-        <v>1027</v>
+        <v>1029</v>
       </c>
       <c r="B273" s="13" t="s">
         <v>25</v>
       </c>
       <c r="C273" s="13" t="s">
-        <v>1028</v>
+        <v>1030</v>
       </c>
       <c r="D273" s="13" t="s">
-        <v>1029</v>
+        <v>1031</v>
       </c>
       <c r="E273" s="13" t="s">
-        <v>1030</v>
+        <v>1032</v>
       </c>
       <c r="F273" s="13" t="s">
-        <v>1031</v>
+        <v>1033</v>
       </c>
       <c r="G273" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H273" s="13">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I273" s="13" t="s">
         <v>1</v>
@@ -12366,28 +12372,28 @@
     </row>
     <row r="274" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A274" s="11" t="s">
-        <v>1032</v>
+        <v>1034</v>
       </c>
       <c r="B274" s="11" t="s">
         <v>26</v>
       </c>
       <c r="C274" s="11" t="s">
-        <v>1033</v>
+        <v>1035</v>
       </c>
       <c r="D274" s="11" t="s">
-        <v>1034</v>
+        <v>1036</v>
       </c>
       <c r="E274" s="11" t="s">
-        <v>1035</v>
+        <v>1037</v>
       </c>
       <c r="F274" s="11" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
       <c r="G274" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H274" s="11">
-        <v>69</v>
+        <v>28</v>
       </c>
       <c r="I274" s="11" t="s">
         <v>1</v>
@@ -12395,28 +12401,28 @@
     </row>
     <row r="275" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A275" s="13" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
       <c r="B275" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C275" s="13" t="s">
-        <v>1038</v>
+        <v>1040</v>
       </c>
       <c r="D275" s="13" t="s">
-        <v>1039</v>
+        <v>1041</v>
       </c>
       <c r="E275" s="13" t="s">
-        <v>1040</v>
+        <v>1042</v>
       </c>
       <c r="F275" s="13" t="s">
-        <v>1041</v>
+        <v>1043</v>
       </c>
       <c r="G275" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H275" s="13">
-        <v>69</v>
+        <v>29</v>
       </c>
       <c r="I275" s="13" t="s">
         <v>1</v>
@@ -12424,19 +12430,19 @@
     </row>
     <row r="276" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A276" s="11" t="s">
-        <v>1042</v>
+        <v>1044</v>
       </c>
       <c r="B276" s="11" t="s">
         <v>26</v>
       </c>
       <c r="C276" s="11" t="s">
-        <v>1043</v>
+        <v>1045</v>
       </c>
       <c r="D276" s="11" t="s">
-        <v>1044</v>
+        <v>1046</v>
       </c>
       <c r="E276" s="11" t="s">
-        <v>1045</v>
+        <v>1047</v>
       </c>
       <c r="F276" s="11" t="s">
         <v>48</v>
@@ -12453,28 +12459,28 @@
     </row>
     <row r="277" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A277" s="13" t="s">
-        <v>1046</v>
+        <v>1048</v>
       </c>
       <c r="B277" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C277" s="13" t="s">
-        <v>1047</v>
+        <v>1049</v>
       </c>
       <c r="D277" s="13" t="s">
-        <v>1048</v>
+        <v>1050</v>
       </c>
       <c r="E277" s="13" t="s">
-        <v>1049</v>
+        <v>1051</v>
       </c>
       <c r="F277" s="13" t="s">
-        <v>1050</v>
+        <v>1052</v>
       </c>
       <c r="G277" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H277" s="13">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="I277" s="13" t="s">
         <v>1</v>
@@ -12482,28 +12488,28 @@
     </row>
     <row r="278" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A278" s="11" t="s">
-        <v>1051</v>
+        <v>1053</v>
       </c>
       <c r="B278" s="11" t="s">
         <v>26</v>
       </c>
       <c r="C278" s="11" t="s">
-        <v>1052</v>
+        <v>1054</v>
       </c>
       <c r="D278" s="11" t="s">
-        <v>1053</v>
+        <v>1055</v>
       </c>
       <c r="E278" s="11" t="s">
-        <v>1054</v>
+        <v>1056</v>
       </c>
       <c r="F278" s="11" t="s">
-        <v>1055</v>
+        <v>1057</v>
       </c>
       <c r="G278" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H278" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I278" s="11" t="s">
         <v>1</v>
@@ -12511,19 +12517,19 @@
     </row>
     <row r="279" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A279" s="13" t="s">
-        <v>1056</v>
+        <v>1058</v>
       </c>
       <c r="B279" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C279" s="13" t="s">
-        <v>1057</v>
+        <v>1059</v>
       </c>
       <c r="D279" s="13" t="s">
-        <v>1058</v>
+        <v>1060</v>
       </c>
       <c r="E279" s="13" t="s">
-        <v>1059</v>
+        <v>1061</v>
       </c>
       <c r="F279" s="13" t="s">
         <v>863</v>
@@ -12532,7 +12538,7 @@
         <v>9</v>
       </c>
       <c r="H279" s="13">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="I279" s="13" t="s">
         <v>1</v>
@@ -12540,28 +12546,28 @@
     </row>
     <row r="280" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A280" s="11" t="s">
-        <v>1060</v>
+        <v>1062</v>
       </c>
       <c r="B280" s="11" t="s">
         <v>26</v>
       </c>
       <c r="C280" s="11" t="s">
-        <v>1061</v>
+        <v>1063</v>
       </c>
       <c r="D280" s="11" t="s">
-        <v>1062</v>
+        <v>1064</v>
       </c>
       <c r="E280" s="11" t="s">
-        <v>1063</v>
+        <v>1065</v>
       </c>
       <c r="F280" s="11" t="s">
-        <v>1064</v>
+        <v>1066</v>
       </c>
       <c r="G280" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H280" s="11">
-        <v>84</v>
+        <v>22</v>
       </c>
       <c r="I280" s="11" t="s">
         <v>1</v>
@@ -12569,28 +12575,28 @@
     </row>
     <row r="281" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A281" s="13" t="s">
-        <v>1065</v>
+        <v>1067</v>
       </c>
       <c r="B281" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C281" s="13" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D281" s="13" t="s">
+        <v>1069</v>
+      </c>
+      <c r="E281" s="13" t="s">
+        <v>1070</v>
+      </c>
+      <c r="F281" s="13" t="s">
         <v>1066</v>
       </c>
-      <c r="D281" s="13" t="s">
-        <v>1067</v>
-      </c>
-      <c r="E281" s="13" t="s">
-        <v>1068</v>
-      </c>
-      <c r="F281" s="13" t="s">
-        <v>1064</v>
-      </c>
       <c r="G281" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H281" s="13">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="I281" s="13" t="s">
         <v>1</v>
@@ -12598,28 +12604,28 @@
     </row>
     <row r="282" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A282" s="11" t="s">
-        <v>1069</v>
+        <v>1071</v>
       </c>
       <c r="B282" s="11" t="s">
         <v>26</v>
       </c>
       <c r="C282" s="11" t="s">
-        <v>1070</v>
+        <v>1072</v>
       </c>
       <c r="D282" s="11" t="s">
-        <v>1071</v>
+        <v>1073</v>
       </c>
       <c r="E282" s="11" t="s">
-        <v>1072</v>
+        <v>1074</v>
       </c>
       <c r="F282" s="11" t="s">
-        <v>1064</v>
+        <v>1066</v>
       </c>
       <c r="G282" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H282" s="11">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="I282" s="11" t="s">
         <v>1</v>
@@ -12627,28 +12633,28 @@
     </row>
     <row r="283" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A283" s="13" t="s">
-        <v>1073</v>
+        <v>1075</v>
       </c>
       <c r="B283" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C283" s="13" t="s">
-        <v>1074</v>
+        <v>1076</v>
       </c>
       <c r="D283" s="13" t="s">
-        <v>1075</v>
+        <v>1077</v>
       </c>
       <c r="E283" s="13" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F283" s="13" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="G283" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H283" s="13">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="I283" s="13" t="s">
         <v>1</v>
@@ -12656,28 +12662,28 @@
     </row>
     <row r="284" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A284" s="11" t="s">
-        <v>1078</v>
+        <v>1080</v>
       </c>
       <c r="B284" s="11" t="s">
         <v>26</v>
       </c>
       <c r="C284" s="11" t="s">
+        <v>1081</v>
+      </c>
+      <c r="D284" s="11" t="s">
+        <v>1082</v>
+      </c>
+      <c r="E284" s="11" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F284" s="11" t="s">
         <v>1079</v>
       </c>
-      <c r="D284" s="11" t="s">
-        <v>1080</v>
-      </c>
-      <c r="E284" s="11" t="s">
-        <v>1076</v>
-      </c>
-      <c r="F284" s="11" t="s">
-        <v>1077</v>
-      </c>
       <c r="G284" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H284" s="11">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="I284" s="11" t="s">
         <v>1</v>
@@ -12685,28 +12691,28 @@
     </row>
     <row r="285" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A285" s="13" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="B285" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C285" s="13" t="s">
-        <v>1082</v>
+        <v>1084</v>
       </c>
       <c r="D285" s="13" t="s">
-        <v>1083</v>
+        <v>1085</v>
       </c>
       <c r="E285" s="13" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F285" s="13" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="G285" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H285" s="13">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="I285" s="13" t="s">
         <v>1</v>
@@ -12714,28 +12720,28 @@
     </row>
     <row r="286" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A286" s="11" t="s">
-        <v>1084</v>
+        <v>1086</v>
       </c>
       <c r="B286" s="11" t="s">
         <v>26</v>
       </c>
       <c r="C286" s="11" t="s">
-        <v>1085</v>
+        <v>1087</v>
       </c>
       <c r="D286" s="11" t="s">
-        <v>1086</v>
+        <v>1088</v>
       </c>
       <c r="E286" s="11" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F286" s="11" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="G286" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H286" s="11">
-        <v>82</v>
+        <v>43</v>
       </c>
       <c r="I286" s="11" t="s">
         <v>1</v>
@@ -12743,28 +12749,28 @@
     </row>
     <row r="287" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A287" s="13" t="s">
-        <v>1087</v>
+        <v>1089</v>
       </c>
       <c r="B287" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C287" s="13" t="s">
-        <v>1088</v>
+        <v>1090</v>
       </c>
       <c r="D287" s="13" t="s">
-        <v>1089</v>
+        <v>1091</v>
       </c>
       <c r="E287" s="13" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F287" s="13" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="G287" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H287" s="13">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I287" s="13" t="s">
         <v>1</v>
@@ -12772,28 +12778,28 @@
     </row>
     <row r="288" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A288" s="11" t="s">
-        <v>1090</v>
+        <v>1092</v>
       </c>
       <c r="B288" s="11" t="s">
         <v>26</v>
       </c>
       <c r="C288" s="11" t="s">
-        <v>1091</v>
+        <v>1093</v>
       </c>
       <c r="D288" s="11" t="s">
-        <v>1092</v>
+        <v>1094</v>
       </c>
       <c r="E288" s="11" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F288" s="11" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="G288" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H288" s="11">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I288" s="11" t="s">
         <v>1</v>
@@ -12801,28 +12807,28 @@
     </row>
     <row r="289" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A289" s="13" t="s">
-        <v>1093</v>
+        <v>1095</v>
       </c>
       <c r="B289" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C289" s="13" t="s">
-        <v>1094</v>
+        <v>1096</v>
       </c>
       <c r="D289" s="13" t="s">
-        <v>1095</v>
+        <v>1097</v>
       </c>
       <c r="E289" s="13" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F289" s="13" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="G289" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H289" s="13">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="I289" s="13" t="s">
         <v>1</v>
@@ -12830,28 +12836,28 @@
     </row>
     <row r="290" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A290" s="11" t="s">
-        <v>1096</v>
+        <v>1098</v>
       </c>
       <c r="B290" s="11" t="s">
         <v>26</v>
       </c>
       <c r="C290" s="11" t="s">
-        <v>1097</v>
+        <v>1099</v>
       </c>
       <c r="D290" s="11" t="s">
-        <v>1098</v>
+        <v>1100</v>
       </c>
       <c r="E290" s="11" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F290" s="11" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="G290" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H290" s="11">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="I290" s="11" t="s">
         <v>1</v>
@@ -12859,28 +12865,28 @@
     </row>
     <row r="291" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A291" s="13" t="s">
-        <v>1099</v>
+        <v>1101</v>
       </c>
       <c r="B291" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C291" s="13" t="s">
-        <v>1100</v>
+        <v>1102</v>
       </c>
       <c r="D291" s="13" t="s">
-        <v>1101</v>
+        <v>1103</v>
       </c>
       <c r="E291" s="13" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F291" s="13" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="G291" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H291" s="13">
-        <v>12</v>
+        <v>84</v>
       </c>
       <c r="I291" s="13" t="s">
         <v>1</v>
@@ -12888,28 +12894,28 @@
     </row>
     <row r="292" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A292" s="11" t="s">
-        <v>1102</v>
+        <v>1104</v>
       </c>
       <c r="B292" s="11" t="s">
         <v>27</v>
       </c>
       <c r="C292" s="11" t="s">
-        <v>1103</v>
+        <v>1105</v>
       </c>
       <c r="D292" s="11" t="s">
-        <v>1072</v>
+        <v>1074</v>
       </c>
       <c r="E292" s="11" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="F292" s="11" t="s">
-        <v>1105</v>
+        <v>1107</v>
       </c>
       <c r="G292" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H292" s="11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I292" s="11" t="s">
         <v>1</v>
@@ -12917,28 +12923,28 @@
     </row>
     <row r="293" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A293" s="13" t="s">
-        <v>1106</v>
+        <v>1108</v>
       </c>
       <c r="B293" s="13" t="s">
         <v>27</v>
       </c>
       <c r="C293" s="13" t="s">
-        <v>1107</v>
+        <v>1109</v>
       </c>
       <c r="D293" s="13" t="s">
-        <v>1108</v>
+        <v>1110</v>
       </c>
       <c r="E293" s="13" t="s">
-        <v>1109</v>
+        <v>1111</v>
       </c>
       <c r="F293" s="13" t="s">
-        <v>1110</v>
+        <v>1112</v>
       </c>
       <c r="G293" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H293" s="13">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="I293" s="13" t="s">
         <v>1</v>
@@ -12946,28 +12952,28 @@
     </row>
     <row r="294" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A294" s="11" t="s">
-        <v>1111</v>
+        <v>1113</v>
       </c>
       <c r="B294" s="11" t="s">
         <v>27</v>
       </c>
       <c r="C294" s="11" t="s">
-        <v>1112</v>
+        <v>1114</v>
       </c>
       <c r="D294" s="11" t="s">
-        <v>1113</v>
+        <v>1115</v>
       </c>
       <c r="E294" s="11" t="s">
-        <v>1114</v>
+        <v>1116</v>
       </c>
       <c r="F294" s="11" t="s">
-        <v>1115</v>
+        <v>1117</v>
       </c>
       <c r="G294" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H294" s="11">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I294" s="11" t="s">
         <v>1</v>
@@ -12975,28 +12981,28 @@
     </row>
     <row r="295" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A295" s="13" t="s">
-        <v>1116</v>
+        <v>1118</v>
       </c>
       <c r="B295" s="13" t="s">
         <v>27</v>
       </c>
       <c r="C295" s="13" t="s">
-        <v>1117</v>
+        <v>1119</v>
       </c>
       <c r="D295" s="13" t="s">
-        <v>1118</v>
+        <v>1120</v>
       </c>
       <c r="E295" s="13" t="s">
-        <v>1119</v>
+        <v>1121</v>
       </c>
       <c r="F295" s="13" t="s">
-        <v>1120</v>
+        <v>1122</v>
       </c>
       <c r="G295" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H295" s="13">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="I295" s="13" t="s">
         <v>1</v>
@@ -13004,28 +13010,28 @@
     </row>
     <row r="296" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A296" s="11" t="s">
-        <v>1121</v>
+        <v>1123</v>
       </c>
       <c r="B296" s="11" t="s">
         <v>28</v>
       </c>
       <c r="C296" s="11" t="s">
-        <v>1122</v>
+        <v>1124</v>
       </c>
       <c r="D296" s="11" t="s">
-        <v>1063</v>
+        <v>1065</v>
       </c>
       <c r="E296" s="11" t="s">
-        <v>1123</v>
+        <v>1125</v>
       </c>
       <c r="F296" s="11" t="s">
-        <v>1124</v>
+        <v>1126</v>
       </c>
       <c r="G296" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H296" s="11">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="I296" s="11" t="s">
         <v>1</v>
@@ -13033,28 +13039,28 @@
     </row>
     <row r="297" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A297" s="13" t="s">
-        <v>1125</v>
+        <v>1127</v>
       </c>
       <c r="B297" s="13" t="s">
         <v>28</v>
       </c>
       <c r="C297" s="13" t="s">
-        <v>1126</v>
+        <v>1128</v>
       </c>
       <c r="D297" s="13" t="s">
-        <v>1127</v>
+        <v>1129</v>
       </c>
       <c r="E297" s="13" t="s">
-        <v>1128</v>
+        <v>1130</v>
       </c>
       <c r="F297" s="13" t="s">
-        <v>1129</v>
+        <v>1131</v>
       </c>
       <c r="G297" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H297" s="13">
-        <v>81</v>
+        <v>49</v>
       </c>
       <c r="I297" s="13" t="s">
         <v>1</v>
@@ -13062,28 +13068,28 @@
     </row>
     <row r="298" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A298" s="11" t="s">
-        <v>1130</v>
+        <v>1132</v>
       </c>
       <c r="B298" s="11" t="s">
         <v>28</v>
       </c>
       <c r="C298" s="11" t="s">
-        <v>1131</v>
+        <v>1133</v>
       </c>
       <c r="D298" s="11" t="s">
-        <v>1132</v>
+        <v>1134</v>
       </c>
       <c r="E298" s="11" t="s">
-        <v>1133</v>
+        <v>1135</v>
       </c>
       <c r="F298" s="11" t="s">
-        <v>1134</v>
+        <v>1136</v>
       </c>
       <c r="G298" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H298" s="11">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I298" s="11" t="s">
         <v>1</v>
@@ -13091,28 +13097,28 @@
     </row>
     <row r="299" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A299" s="13" t="s">
-        <v>1135</v>
+        <v>1137</v>
       </c>
       <c r="B299" s="13" t="s">
         <v>29</v>
       </c>
       <c r="C299" s="13" t="s">
-        <v>1136</v>
+        <v>1138</v>
       </c>
       <c r="D299" s="13" t="s">
-        <v>1068</v>
+        <v>1070</v>
       </c>
       <c r="E299" s="13" t="s">
-        <v>1137</v>
+        <v>1139</v>
       </c>
       <c r="F299" s="13" t="s">
-        <v>1124</v>
+        <v>1126</v>
       </c>
       <c r="G299" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H299" s="13">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="I299" s="13" t="s">
         <v>1</v>
@@ -13120,28 +13126,28 @@
     </row>
     <row r="300" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A300" s="11" t="s">
-        <v>1138</v>
+        <v>1140</v>
       </c>
       <c r="B300" s="11" t="s">
         <v>29</v>
       </c>
       <c r="C300" s="11" t="s">
-        <v>1139</v>
+        <v>1141</v>
       </c>
       <c r="D300" s="11" t="s">
-        <v>1140</v>
+        <v>1142</v>
       </c>
       <c r="E300" s="11" t="s">
-        <v>1141</v>
+        <v>1143</v>
       </c>
       <c r="F300" s="11" t="s">
-        <v>1129</v>
+        <v>1131</v>
       </c>
       <c r="G300" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H300" s="11">
-        <v>89</v>
+        <v>18</v>
       </c>
       <c r="I300" s="11" t="s">
         <v>1</v>
@@ -13149,28 +13155,28 @@
     </row>
     <row r="301" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A301" s="13" t="s">
-        <v>1142</v>
+        <v>1144</v>
       </c>
       <c r="B301" s="13" t="s">
         <v>29</v>
       </c>
       <c r="C301" s="13" t="s">
-        <v>1143</v>
+        <v>1145</v>
       </c>
       <c r="D301" s="13" t="s">
-        <v>1132</v>
+        <v>1134</v>
       </c>
       <c r="E301" s="13" t="s">
-        <v>1133</v>
+        <v>1135</v>
       </c>
       <c r="F301" s="13" t="s">
-        <v>1134</v>
+        <v>1136</v>
       </c>
       <c r="G301" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H301" s="13">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I301" s="13" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
test: run appium-tests and update report
</commit_message>
<xml_diff>
--- a/testing/appium-tests/Test_Report.xlsx
+++ b/testing/appium-tests/Test_Report.xlsx
@@ -1391,7 +1391,7 @@
     <t>TestCase_Sales_15: Submit random sales variation 15</t>
   </si>
   <si>
-    <t>Item: "Item 1", Quantity: 126, Date: Today</t>
+    <t>Item: "Item 1", Quantity: 148, Date: Today</t>
   </si>
   <si>
     <t>Sales record saved and threshold check triggered</t>
@@ -1406,7 +1406,7 @@
     <t>TestCase_Sales_16: Submit random sales variation 16</t>
   </si>
   <si>
-    <t>Item: "Item 2", Quantity: 131, Date: Today</t>
+    <t>Item: "Item 2", Quantity: 79, Date: Today</t>
   </si>
   <si>
     <t>TC111</t>
@@ -1415,7 +1415,7 @@
     <t>TestCase_Sales_17: Submit random sales variation 17</t>
   </si>
   <si>
-    <t>Item: "Item 3", Quantity: 111, Date: Today</t>
+    <t>Item: "Item 3", Quantity: 153, Date: Today</t>
   </si>
   <si>
     <t>TC112</t>
@@ -1424,7 +1424,7 @@
     <t>TestCase_Sales_18: Submit random sales variation 18</t>
   </si>
   <si>
-    <t>Item: "Item 4", Quantity: 53, Date: Today</t>
+    <t>Item: "Item 4", Quantity: 105, Date: Today</t>
   </si>
   <si>
     <t>TC113</t>
@@ -1433,7 +1433,7 @@
     <t>TestCase_Sales_19: Submit random sales variation 19</t>
   </si>
   <si>
-    <t>Item: "Item 5", Quantity: 73, Date: Today</t>
+    <t>Item: "Item 5", Quantity: 192, Date: Today</t>
   </si>
   <si>
     <t>TC114</t>
@@ -1442,7 +1442,7 @@
     <t>TestCase_Sales_20: Submit random sales variation 20</t>
   </si>
   <si>
-    <t>Item: "Item 1", Quantity: 100, Date: Today</t>
+    <t>Item: "Item 1", Quantity: 191, Date: Today</t>
   </si>
   <si>
     <t>TC115</t>
@@ -1451,7 +1451,7 @@
     <t>TestCase_Sales_21: Submit random sales variation 21</t>
   </si>
   <si>
-    <t>Item: "Item 2", Quantity: 112, Date: Today</t>
+    <t>Item: "Item 2", Quantity: 113, Date: Today</t>
   </si>
   <si>
     <t>TC116</t>
@@ -1460,7 +1460,7 @@
     <t>TestCase_Sales_22: Submit random sales variation 22</t>
   </si>
   <si>
-    <t>Item: "Item 3", Quantity: 180, Date: Today</t>
+    <t>Item: "Item 3", Quantity: 78, Date: Today</t>
   </si>
   <si>
     <t>TC117</t>
@@ -1469,7 +1469,7 @@
     <t>TestCase_Sales_23: Submit random sales variation 23</t>
   </si>
   <si>
-    <t>Item: "Item 4", Quantity: 29, Date: Today</t>
+    <t>Item: "Item 4", Quantity: 161, Date: Today</t>
   </si>
   <si>
     <t>TC118</t>
@@ -1478,7 +1478,7 @@
     <t>TestCase_Sales_24: Submit random sales variation 24</t>
   </si>
   <si>
-    <t>Item: "Item 5", Quantity: 110, Date: Today</t>
+    <t>Item: "Item 5", Quantity: 182, Date: Today</t>
   </si>
   <si>
     <t>TC119</t>
@@ -1487,7 +1487,7 @@
     <t>TestCase_Sales_25: Submit random sales variation 25</t>
   </si>
   <si>
-    <t>Item: "Item 1", Quantity: 68, Date: Today</t>
+    <t>Item: "Item 1", Quantity: 194, Date: Today</t>
   </si>
   <si>
     <t>TC120</t>
@@ -1496,7 +1496,7 @@
     <t>TestCase_Sales_26: Submit random sales variation 26</t>
   </si>
   <si>
-    <t>Item: "Item 2", Quantity: 87, Date: Today</t>
+    <t>Item: "Item 2", Quantity: 139, Date: Today</t>
   </si>
   <si>
     <t>TC121</t>
@@ -1505,7 +1505,7 @@
     <t>TestCase_Sales_27: Submit random sales variation 27</t>
   </si>
   <si>
-    <t>Item: "Item 3", Quantity: 17, Date: Today</t>
+    <t>Item: "Item 3", Quantity: 20, Date: Today</t>
   </si>
   <si>
     <t>TC122</t>
@@ -1514,196 +1514,196 @@
     <t>TestCase_Sales_28: Submit random sales variation 28</t>
   </si>
   <si>
+    <t>Item: "Item 4", Quantity: 110, Date: Today</t>
+  </si>
+  <si>
+    <t>TC123</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_29: Submit random sales variation 29</t>
+  </si>
+  <si>
+    <t>Item: "Item 5", Quantity: 93, Date: Today</t>
+  </si>
+  <si>
+    <t>TC124</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_30: Submit random sales variation 30</t>
+  </si>
+  <si>
+    <t>Item: "Item 1", Quantity: 105, Date: Today</t>
+  </si>
+  <si>
+    <t>TC125</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_31: Submit random sales variation 31</t>
+  </si>
+  <si>
+    <t>Item: "Item 2", Quantity: 23, Date: Today</t>
+  </si>
+  <si>
+    <t>TC126</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_32: Submit random sales variation 32</t>
+  </si>
+  <si>
+    <t>Item: "Item 3", Quantity: 65, Date: Today</t>
+  </si>
+  <si>
+    <t>TC127</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_33: Submit random sales variation 33</t>
+  </si>
+  <si>
+    <t>Item: "Item 4", Quantity: 135, Date: Today</t>
+  </si>
+  <si>
+    <t>TC128</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_34: Submit random sales variation 34</t>
+  </si>
+  <si>
+    <t>Item: "Item 5", Quantity: 156, Date: Today</t>
+  </si>
+  <si>
+    <t>TC129</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_35: Submit random sales variation 35</t>
+  </si>
+  <si>
+    <t>Item: "Item 1", Quantity: 70, Date: Today</t>
+  </si>
+  <si>
+    <t>TC130</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_36: Submit random sales variation 36</t>
+  </si>
+  <si>
+    <t>Item: "Item 2", Quantity: 143, Date: Today</t>
+  </si>
+  <si>
+    <t>TC131</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_37: Submit random sales variation 37</t>
+  </si>
+  <si>
+    <t>Item: "Item 3", Quantity: 105, Date: Today</t>
+  </si>
+  <si>
+    <t>TC132</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_38: Submit random sales variation 38</t>
+  </si>
+  <si>
+    <t>Item: "Item 4", Quantity: 198, Date: Today</t>
+  </si>
+  <si>
+    <t>TC133</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_39: Submit random sales variation 39</t>
+  </si>
+  <si>
+    <t>Item: "Item 5", Quantity: 108, Date: Today</t>
+  </si>
+  <si>
+    <t>TC134</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_40: Submit random sales variation 40</t>
+  </si>
+  <si>
+    <t>Item: "Item 1", Quantity: 5, Date: Today</t>
+  </si>
+  <si>
+    <t>TC135</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_41: Submit random sales variation 41</t>
+  </si>
+  <si>
+    <t>Item: "Item 2", Quantity: 25, Date: Today</t>
+  </si>
+  <si>
+    <t>TC136</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_42: Submit random sales variation 42</t>
+  </si>
+  <si>
+    <t>Item: "Item 3", Quantity: 173, Date: Today</t>
+  </si>
+  <si>
+    <t>TC137</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_43: Submit random sales variation 43</t>
+  </si>
+  <si>
+    <t>Item: "Item 4", Quantity: 14, Date: Today</t>
+  </si>
+  <si>
+    <t>TC138</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_44: Submit random sales variation 44</t>
+  </si>
+  <si>
+    <t>Item: "Item 5", Quantity: 91, Date: Today</t>
+  </si>
+  <si>
+    <t>TC139</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_45: Submit random sales variation 45</t>
+  </si>
+  <si>
+    <t>Item: "Item 1", Quantity: 152, Date: Today</t>
+  </si>
+  <si>
+    <t>TC140</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_46: Submit random sales variation 46</t>
+  </si>
+  <si>
+    <t>Item: "Item 2", Quantity: 47, Date: Today</t>
+  </si>
+  <si>
+    <t>TC141</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_47: Submit random sales variation 47</t>
+  </si>
+  <si>
+    <t>Item: "Item 3", Quantity: 161, Date: Today</t>
+  </si>
+  <si>
+    <t>TC142</t>
+  </si>
+  <si>
+    <t>TestCase_Sales_48: Submit random sales variation 48</t>
+  </si>
+  <si>
     <t>Item: "Item 4", Quantity: 178, Date: Today</t>
   </si>
   <si>
-    <t>TC123</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_29: Submit random sales variation 29</t>
-  </si>
-  <si>
-    <t>Item: "Item 5", Quantity: 52, Date: Today</t>
-  </si>
-  <si>
-    <t>TC124</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_30: Submit random sales variation 30</t>
-  </si>
-  <si>
-    <t>Item: "Item 1", Quantity: 78, Date: Today</t>
-  </si>
-  <si>
-    <t>TC125</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_31: Submit random sales variation 31</t>
-  </si>
-  <si>
-    <t>Item: "Item 2", Quantity: 88, Date: Today</t>
-  </si>
-  <si>
-    <t>TC126</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_32: Submit random sales variation 32</t>
-  </si>
-  <si>
-    <t>Item: "Item 3", Quantity: 80, Date: Today</t>
-  </si>
-  <si>
-    <t>TC127</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_33: Submit random sales variation 33</t>
-  </si>
-  <si>
-    <t>Item: "Item 4", Quantity: 46, Date: Today</t>
-  </si>
-  <si>
-    <t>TC128</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_34: Submit random sales variation 34</t>
-  </si>
-  <si>
-    <t>Item: "Item 5", Quantity: 12, Date: Today</t>
-  </si>
-  <si>
-    <t>TC129</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_35: Submit random sales variation 35</t>
-  </si>
-  <si>
-    <t>Item: "Item 1", Quantity: 4, Date: Today</t>
-  </si>
-  <si>
-    <t>TC130</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_36: Submit random sales variation 36</t>
-  </si>
-  <si>
-    <t>Item: "Item 2", Quantity: 143, Date: Today</t>
-  </si>
-  <si>
-    <t>TC131</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_37: Submit random sales variation 37</t>
-  </si>
-  <si>
-    <t>Item: "Item 3", Quantity: 133, Date: Today</t>
-  </si>
-  <si>
-    <t>TC132</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_38: Submit random sales variation 38</t>
-  </si>
-  <si>
-    <t>Item: "Item 4", Quantity: 32, Date: Today</t>
-  </si>
-  <si>
-    <t>TC133</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_39: Submit random sales variation 39</t>
-  </si>
-  <si>
-    <t>Item: "Item 5", Quantity: 24, Date: Today</t>
-  </si>
-  <si>
-    <t>TC134</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_40: Submit random sales variation 40</t>
-  </si>
-  <si>
-    <t>Item: "Item 1", Quantity: 39, Date: Today</t>
-  </si>
-  <si>
-    <t>TC135</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_41: Submit random sales variation 41</t>
-  </si>
-  <si>
-    <t>Item: "Item 2", Quantity: 79, Date: Today</t>
-  </si>
-  <si>
-    <t>TC136</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_42: Submit random sales variation 42</t>
-  </si>
-  <si>
-    <t>Item: "Item 3", Quantity: 188, Date: Today</t>
-  </si>
-  <si>
-    <t>TC137</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_43: Submit random sales variation 43</t>
-  </si>
-  <si>
-    <t>Item: "Item 4", Quantity: 159, Date: Today</t>
-  </si>
-  <si>
-    <t>TC138</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_44: Submit random sales variation 44</t>
-  </si>
-  <si>
-    <t>Item: "Item 5", Quantity: 48, Date: Today</t>
-  </si>
-  <si>
-    <t>TC139</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_45: Submit random sales variation 45</t>
-  </si>
-  <si>
-    <t>Item: "Item 1", Quantity: 55, Date: Today</t>
-  </si>
-  <si>
-    <t>TC140</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_46: Submit random sales variation 46</t>
-  </si>
-  <si>
-    <t>Item: "Item 2", Quantity: 65, Date: Today</t>
-  </si>
-  <si>
-    <t>TC141</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_47: Submit random sales variation 47</t>
-  </si>
-  <si>
-    <t>Item: "Item 3", Quantity: 140, Date: Today</t>
-  </si>
-  <si>
-    <t>TC142</t>
-  </si>
-  <si>
-    <t>TestCase_Sales_48: Submit random sales variation 48</t>
-  </si>
-  <si>
-    <t>Item: "Item 4", Quantity: 192, Date: Today</t>
-  </si>
-  <si>
     <t>TC143</t>
   </si>
   <si>
     <t>TestCase_Sales_49: Submit random sales variation 49</t>
   </si>
   <si>
-    <t>Item: "Item 5", Quantity: 164, Date: Today</t>
+    <t>Item: "Item 5", Quantity: 131, Date: Today</t>
   </si>
   <si>
     <t>TC144</t>
@@ -1712,7 +1712,7 @@
     <t>TestCase_Sales_50: Submit random sales variation 50</t>
   </si>
   <si>
-    <t>Item: "Item 1", Quantity: 60, Date: Today</t>
+    <t>Item: "Item 1", Quantity: 37, Date: Today</t>
   </si>
   <si>
     <t>TC145</t>
@@ -2876,151 +2876,151 @@
     <t>TC251</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_09: Score 21 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 21</t>
+    <t>TestCase_HealthScore_09: Score 97 shows "Thriving" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 97</t>
+  </si>
+  <si>
+    <t>Verdict: "Thriving" displayed</t>
+  </si>
+  <si>
+    <t>Verdict matched expected business logic</t>
+  </si>
+  <si>
+    <t>TC252</t>
+  </si>
+  <si>
+    <t>TestCase_HealthScore_10: Score 75 shows "Work in Progress" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 75</t>
+  </si>
+  <si>
+    <t>Verdict: "Work in Progress" displayed</t>
+  </si>
+  <si>
+    <t>TC253</t>
+  </si>
+  <si>
+    <t>TestCase_HealthScore_11: Score 92 shows "Thriving" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 92</t>
+  </si>
+  <si>
+    <t>TC254</t>
+  </si>
+  <si>
+    <t>TestCase_HealthScore_12: Score 49 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 49</t>
   </si>
   <si>
     <t>Verdict: "Immediate Action Needed" displayed</t>
   </si>
   <si>
-    <t>Verdict matched expected business logic</t>
-  </si>
-  <si>
-    <t>TC252</t>
-  </si>
-  <si>
-    <t>TestCase_HealthScore_10: Score 16 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 16</t>
-  </si>
-  <si>
-    <t>TC253</t>
-  </si>
-  <si>
-    <t>TestCase_HealthScore_11: Score 94 shows "Thriving" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 94</t>
-  </si>
-  <si>
-    <t>Verdict: "Thriving" displayed</t>
-  </si>
-  <si>
-    <t>TC254</t>
-  </si>
-  <si>
-    <t>TestCase_HealthScore_12: Score 54 shows "Work in Progress" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 54</t>
-  </si>
-  <si>
-    <t>Verdict: "Work in Progress" displayed</t>
-  </si>
-  <si>
     <t>TC255</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_13: Score 86 shows "Thriving" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 86</t>
+    <t>TestCase_HealthScore_13: Score 82 shows "Thriving" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 82</t>
   </si>
   <si>
     <t>TC256</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_14: Score 24 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 24</t>
+    <t>TestCase_HealthScore_14: Score 10 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 10</t>
   </si>
   <si>
     <t>TC257</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_15: Score 72 shows "Work in Progress" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 72</t>
+    <t>TestCase_HealthScore_15: Score 42 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 42</t>
   </si>
   <si>
     <t>TC258</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_16: Score 15 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 15</t>
+    <t>TestCase_HealthScore_16: Score 49 shows "Immediate Action Needed" verdict</t>
   </si>
   <si>
     <t>TC259</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_17: Score 16 shows "Immediate Action Needed" verdict</t>
+    <t>TestCase_HealthScore_17: Score 31 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 31</t>
   </si>
   <si>
     <t>TC260</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_18: Score 16 shows "Immediate Action Needed" verdict</t>
+    <t>TestCase_HealthScore_18: Score 41 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 41</t>
   </si>
   <si>
     <t>TC261</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_19: Score 81 shows "Thriving" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 81</t>
+    <t>TestCase_HealthScore_19: Score 5 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 5</t>
   </si>
   <si>
     <t>TC262</t>
   </si>
   <si>
-    <t>TestCase_HealthScore_20: Score 89 shows "Thriving" verdict</t>
+    <t>TestCase_HealthScore_20: Score 82 shows "Thriving" verdict</t>
+  </si>
+  <si>
+    <t>TC263</t>
+  </si>
+  <si>
+    <t>TestCase_HealthScore_21: Score 83 shows "Thriving" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 83</t>
+  </si>
+  <si>
+    <t>TC264</t>
+  </si>
+  <si>
+    <t>TestCase_HealthScore_22: Score 89 shows "Thriving" verdict</t>
   </si>
   <si>
     <t>Simulated score: 89</t>
   </si>
   <si>
-    <t>TC263</t>
-  </si>
-  <si>
-    <t>TestCase_HealthScore_21: Score 3 shows "Immediate Action Needed" verdict</t>
+    <t>TC265</t>
+  </si>
+  <si>
+    <t>TestCase_HealthScore_23: Score 14 shows "Immediate Action Needed" verdict</t>
+  </si>
+  <si>
+    <t>Simulated score: 14</t>
+  </si>
+  <si>
+    <t>TC266</t>
+  </si>
+  <si>
+    <t>TestCase_HealthScore_24: Score 3 shows "Immediate Action Needed" verdict</t>
   </si>
   <si>
     <t>Simulated score: 3</t>
-  </si>
-  <si>
-    <t>TC264</t>
-  </si>
-  <si>
-    <t>TestCase_HealthScore_22: Score 88 shows "Thriving" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 88</t>
-  </si>
-  <si>
-    <t>TC265</t>
-  </si>
-  <si>
-    <t>TestCase_HealthScore_23: Score 5 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 5</t>
-  </si>
-  <si>
-    <t>TC266</t>
-  </si>
-  <si>
-    <t>TestCase_HealthScore_24: Score 37 shows "Immediate Action Needed" verdict</t>
-  </si>
-  <si>
-    <t>Simulated score: 37</t>
   </si>
   <si>
     <t>TC267</t>
@@ -4502,7 +4502,7 @@
         <v>9</v>
       </c>
       <c r="H2" s="11">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="I2" s="11" t="s">
         <v>1</v>
@@ -4531,7 +4531,7 @@
         <v>9</v>
       </c>
       <c r="H3" s="13">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="I3" s="13" t="s">
         <v>1</v>
@@ -4560,7 +4560,7 @@
         <v>9</v>
       </c>
       <c r="H4" s="11">
-        <v>14</v>
+        <v>66</v>
       </c>
       <c r="I4" s="11" t="s">
         <v>1</v>
@@ -4589,7 +4589,7 @@
         <v>9</v>
       </c>
       <c r="H5" s="13">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I5" s="13" t="s">
         <v>1</v>
@@ -4618,7 +4618,7 @@
         <v>9</v>
       </c>
       <c r="H6" s="11">
-        <v>71</v>
+        <v>14</v>
       </c>
       <c r="I6" s="11" t="s">
         <v>1</v>
@@ -4647,7 +4647,7 @@
         <v>9</v>
       </c>
       <c r="H7" s="13">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="I7" s="13" t="s">
         <v>1</v>
@@ -4705,7 +4705,7 @@
         <v>9</v>
       </c>
       <c r="H9" s="13">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="I9" s="13" t="s">
         <v>1</v>
@@ -4734,7 +4734,7 @@
         <v>9</v>
       </c>
       <c r="H10" s="11">
-        <v>55</v>
+        <v>83</v>
       </c>
       <c r="I10" s="11" t="s">
         <v>1</v>
@@ -4763,7 +4763,7 @@
         <v>9</v>
       </c>
       <c r="H11" s="13">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="I11" s="13" t="s">
         <v>1</v>
@@ -4792,7 +4792,7 @@
         <v>9</v>
       </c>
       <c r="H12" s="11">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="I12" s="11" t="s">
         <v>1</v>
@@ -4821,7 +4821,7 @@
         <v>9</v>
       </c>
       <c r="H13" s="13">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="I13" s="13" t="s">
         <v>1</v>
@@ -4850,7 +4850,7 @@
         <v>9</v>
       </c>
       <c r="H14" s="11">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="I14" s="11" t="s">
         <v>1</v>
@@ -4879,7 +4879,7 @@
         <v>9</v>
       </c>
       <c r="H15" s="13">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="I15" s="13" t="s">
         <v>1</v>
@@ -4908,7 +4908,7 @@
         <v>9</v>
       </c>
       <c r="H16" s="11">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="I16" s="11" t="s">
         <v>1</v>
@@ -4937,7 +4937,7 @@
         <v>9</v>
       </c>
       <c r="H17" s="13">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="I17" s="13" t="s">
         <v>1</v>
@@ -4966,7 +4966,7 @@
         <v>9</v>
       </c>
       <c r="H18" s="11">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I18" s="11" t="s">
         <v>1</v>
@@ -4995,7 +4995,7 @@
         <v>9</v>
       </c>
       <c r="H19" s="13">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I19" s="13" t="s">
         <v>1</v>
@@ -5024,7 +5024,7 @@
         <v>9</v>
       </c>
       <c r="H20" s="11">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I20" s="11" t="s">
         <v>1</v>
@@ -5053,7 +5053,7 @@
         <v>9</v>
       </c>
       <c r="H21" s="13">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="I21" s="13" t="s">
         <v>1</v>
@@ -5082,7 +5082,7 @@
         <v>9</v>
       </c>
       <c r="H22" s="11">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="I22" s="11" t="s">
         <v>1</v>
@@ -5111,7 +5111,7 @@
         <v>9</v>
       </c>
       <c r="H23" s="13">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="I23" s="13" t="s">
         <v>1</v>
@@ -5140,7 +5140,7 @@
         <v>9</v>
       </c>
       <c r="H24" s="11">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="I24" s="11" t="s">
         <v>1</v>
@@ -5169,7 +5169,7 @@
         <v>9</v>
       </c>
       <c r="H25" s="13">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="I25" s="13" t="s">
         <v>1</v>
@@ -5198,7 +5198,7 @@
         <v>9</v>
       </c>
       <c r="H26" s="11">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="I26" s="11" t="s">
         <v>1</v>
@@ -5227,7 +5227,7 @@
         <v>9</v>
       </c>
       <c r="H27" s="13">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="I27" s="13" t="s">
         <v>1</v>
@@ -5256,7 +5256,7 @@
         <v>9</v>
       </c>
       <c r="H28" s="11">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="I28" s="11" t="s">
         <v>1</v>
@@ -5285,7 +5285,7 @@
         <v>9</v>
       </c>
       <c r="H29" s="13">
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="I29" s="13" t="s">
         <v>1</v>
@@ -5314,7 +5314,7 @@
         <v>9</v>
       </c>
       <c r="H30" s="11">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="I30" s="11" t="s">
         <v>1</v>
@@ -5343,7 +5343,7 @@
         <v>9</v>
       </c>
       <c r="H31" s="13">
-        <v>39</v>
+        <v>63</v>
       </c>
       <c r="I31" s="13" t="s">
         <v>1</v>
@@ -5372,7 +5372,7 @@
         <v>9</v>
       </c>
       <c r="H32" s="11">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="I32" s="11" t="s">
         <v>1</v>
@@ -5401,7 +5401,7 @@
         <v>9</v>
       </c>
       <c r="H33" s="13">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="I33" s="13" t="s">
         <v>1</v>
@@ -5430,7 +5430,7 @@
         <v>9</v>
       </c>
       <c r="H34" s="11">
-        <v>30</v>
+        <v>87</v>
       </c>
       <c r="I34" s="11" t="s">
         <v>1</v>
@@ -5459,7 +5459,7 @@
         <v>9</v>
       </c>
       <c r="H35" s="13">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="I35" s="13" t="s">
         <v>1</v>
@@ -5488,7 +5488,7 @@
         <v>9</v>
       </c>
       <c r="H36" s="11">
-        <v>26</v>
+        <v>82</v>
       </c>
       <c r="I36" s="11" t="s">
         <v>1</v>
@@ -5517,7 +5517,7 @@
         <v>9</v>
       </c>
       <c r="H37" s="13">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="I37" s="13" t="s">
         <v>1</v>
@@ -5546,7 +5546,7 @@
         <v>9</v>
       </c>
       <c r="H38" s="11">
-        <v>64</v>
+        <v>24</v>
       </c>
       <c r="I38" s="11" t="s">
         <v>1</v>
@@ -5575,7 +5575,7 @@
         <v>9</v>
       </c>
       <c r="H39" s="13">
-        <v>62</v>
+        <v>84</v>
       </c>
       <c r="I39" s="13" t="s">
         <v>1</v>
@@ -5604,7 +5604,7 @@
         <v>9</v>
       </c>
       <c r="H40" s="11">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="I40" s="11" t="s">
         <v>1</v>
@@ -5633,7 +5633,7 @@
         <v>9</v>
       </c>
       <c r="H41" s="13">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="I41" s="13" t="s">
         <v>1</v>
@@ -5662,7 +5662,7 @@
         <v>9</v>
       </c>
       <c r="H42" s="11">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="I42" s="11" t="s">
         <v>1</v>
@@ -5691,7 +5691,7 @@
         <v>9</v>
       </c>
       <c r="H43" s="13">
-        <v>73</v>
+        <v>12</v>
       </c>
       <c r="I43" s="13" t="s">
         <v>1</v>
@@ -5720,7 +5720,7 @@
         <v>9</v>
       </c>
       <c r="H44" s="11">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="I44" s="11" t="s">
         <v>1</v>
@@ -5749,7 +5749,7 @@
         <v>9</v>
       </c>
       <c r="H45" s="13">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="I45" s="13" t="s">
         <v>1</v>
@@ -5778,7 +5778,7 @@
         <v>9</v>
       </c>
       <c r="H46" s="11">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="I46" s="11" t="s">
         <v>1</v>
@@ -5807,7 +5807,7 @@
         <v>9</v>
       </c>
       <c r="H47" s="13">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="I47" s="13" t="s">
         <v>1</v>
@@ -5836,7 +5836,7 @@
         <v>9</v>
       </c>
       <c r="H48" s="11">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="I48" s="11" t="s">
         <v>1</v>
@@ -5865,7 +5865,7 @@
         <v>9</v>
       </c>
       <c r="H49" s="13">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="I49" s="13" t="s">
         <v>1</v>
@@ -5894,7 +5894,7 @@
         <v>9</v>
       </c>
       <c r="H50" s="11">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="I50" s="11" t="s">
         <v>1</v>
@@ -5923,7 +5923,7 @@
         <v>9</v>
       </c>
       <c r="H51" s="13">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="I51" s="13" t="s">
         <v>1</v>
@@ -5952,7 +5952,7 @@
         <v>9</v>
       </c>
       <c r="H52" s="11">
-        <v>81</v>
+        <v>48</v>
       </c>
       <c r="I52" s="11" t="s">
         <v>1</v>
@@ -5981,7 +5981,7 @@
         <v>9</v>
       </c>
       <c r="H53" s="13">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="I53" s="13" t="s">
         <v>1</v>
@@ -6010,7 +6010,7 @@
         <v>9</v>
       </c>
       <c r="H54" s="11">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="I54" s="11" t="s">
         <v>1</v>
@@ -6039,7 +6039,7 @@
         <v>9</v>
       </c>
       <c r="H55" s="13">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="I55" s="13" t="s">
         <v>1</v>
@@ -6097,7 +6097,7 @@
         <v>9</v>
       </c>
       <c r="H57" s="13">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="I57" s="13" t="s">
         <v>1</v>
@@ -6126,7 +6126,7 @@
         <v>9</v>
       </c>
       <c r="H58" s="11">
-        <v>80</v>
+        <v>24</v>
       </c>
       <c r="I58" s="11" t="s">
         <v>1</v>
@@ -6155,7 +6155,7 @@
         <v>9</v>
       </c>
       <c r="H59" s="13">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="I59" s="13" t="s">
         <v>1</v>
@@ -6184,7 +6184,7 @@
         <v>9</v>
       </c>
       <c r="H60" s="11">
-        <v>88</v>
+        <v>66</v>
       </c>
       <c r="I60" s="11" t="s">
         <v>1</v>
@@ -6213,7 +6213,7 @@
         <v>9</v>
       </c>
       <c r="H61" s="13">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I61" s="13" t="s">
         <v>1</v>
@@ -6242,7 +6242,7 @@
         <v>9</v>
       </c>
       <c r="H62" s="11">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="I62" s="11" t="s">
         <v>1</v>
@@ -6271,7 +6271,7 @@
         <v>9</v>
       </c>
       <c r="H63" s="13">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="I63" s="13" t="s">
         <v>1</v>
@@ -6300,7 +6300,7 @@
         <v>9</v>
       </c>
       <c r="H64" s="11">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="I64" s="11" t="s">
         <v>1</v>
@@ -6329,7 +6329,7 @@
         <v>9</v>
       </c>
       <c r="H65" s="13">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="I65" s="13" t="s">
         <v>1</v>
@@ -6358,7 +6358,7 @@
         <v>9</v>
       </c>
       <c r="H66" s="11">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="I66" s="11" t="s">
         <v>1</v>
@@ -6387,7 +6387,7 @@
         <v>9</v>
       </c>
       <c r="H67" s="13">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="I67" s="13" t="s">
         <v>1</v>
@@ -6416,7 +6416,7 @@
         <v>9</v>
       </c>
       <c r="H68" s="11">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="I68" s="11" t="s">
         <v>1</v>
@@ -6445,7 +6445,7 @@
         <v>9</v>
       </c>
       <c r="H69" s="13">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="I69" s="13" t="s">
         <v>1</v>
@@ -6474,7 +6474,7 @@
         <v>9</v>
       </c>
       <c r="H70" s="11">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="I70" s="11" t="s">
         <v>1</v>
@@ -6503,7 +6503,7 @@
         <v>9</v>
       </c>
       <c r="H71" s="13">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="I71" s="13" t="s">
         <v>1</v>
@@ -6532,7 +6532,7 @@
         <v>9</v>
       </c>
       <c r="H72" s="11">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I72" s="11" t="s">
         <v>1</v>
@@ -6561,7 +6561,7 @@
         <v>9</v>
       </c>
       <c r="H73" s="13">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="I73" s="13" t="s">
         <v>1</v>
@@ -6590,7 +6590,7 @@
         <v>9</v>
       </c>
       <c r="H74" s="11">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="I74" s="11" t="s">
         <v>1</v>
@@ -6619,7 +6619,7 @@
         <v>9</v>
       </c>
       <c r="H75" s="13">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="I75" s="13" t="s">
         <v>1</v>
@@ -6648,7 +6648,7 @@
         <v>9</v>
       </c>
       <c r="H76" s="11">
-        <v>57</v>
+        <v>86</v>
       </c>
       <c r="I76" s="11" t="s">
         <v>1</v>
@@ -6677,7 +6677,7 @@
         <v>9</v>
       </c>
       <c r="H77" s="13">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="I77" s="13" t="s">
         <v>1</v>
@@ -6706,7 +6706,7 @@
         <v>9</v>
       </c>
       <c r="H78" s="11">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="I78" s="11" t="s">
         <v>1</v>
@@ -6735,7 +6735,7 @@
         <v>9</v>
       </c>
       <c r="H79" s="13">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="I79" s="13" t="s">
         <v>1</v>
@@ -6764,7 +6764,7 @@
         <v>9</v>
       </c>
       <c r="H80" s="11">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="I80" s="11" t="s">
         <v>1</v>
@@ -6793,7 +6793,7 @@
         <v>9</v>
       </c>
       <c r="H81" s="13">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="I81" s="13" t="s">
         <v>1</v>
@@ -6822,7 +6822,7 @@
         <v>9</v>
       </c>
       <c r="H82" s="11">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="I82" s="11" t="s">
         <v>1</v>
@@ -6851,7 +6851,7 @@
         <v>9</v>
       </c>
       <c r="H83" s="13">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="I83" s="13" t="s">
         <v>1</v>
@@ -6880,7 +6880,7 @@
         <v>9</v>
       </c>
       <c r="H84" s="11">
-        <v>66</v>
+        <v>14</v>
       </c>
       <c r="I84" s="11" t="s">
         <v>1</v>
@@ -6909,7 +6909,7 @@
         <v>9</v>
       </c>
       <c r="H85" s="13">
-        <v>77</v>
+        <v>41</v>
       </c>
       <c r="I85" s="13" t="s">
         <v>1</v>
@@ -6938,7 +6938,7 @@
         <v>9</v>
       </c>
       <c r="H86" s="11">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I86" s="11" t="s">
         <v>1</v>
@@ -6967,7 +6967,7 @@
         <v>9</v>
       </c>
       <c r="H87" s="13">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="I87" s="13" t="s">
         <v>1</v>
@@ -6996,7 +6996,7 @@
         <v>9</v>
       </c>
       <c r="H88" s="11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I88" s="11" t="s">
         <v>1</v>
@@ -7025,7 +7025,7 @@
         <v>9</v>
       </c>
       <c r="H89" s="13">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="I89" s="13" t="s">
         <v>1</v>
@@ -7054,7 +7054,7 @@
         <v>9</v>
       </c>
       <c r="H90" s="11">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="I90" s="11" t="s">
         <v>1</v>
@@ -7083,7 +7083,7 @@
         <v>9</v>
       </c>
       <c r="H91" s="13">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="I91" s="13" t="s">
         <v>1</v>
@@ -7112,7 +7112,7 @@
         <v>9</v>
       </c>
       <c r="H92" s="11">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="I92" s="11" t="s">
         <v>1</v>
@@ -7141,7 +7141,7 @@
         <v>9</v>
       </c>
       <c r="H93" s="13">
-        <v>89</v>
+        <v>35</v>
       </c>
       <c r="I93" s="13" t="s">
         <v>1</v>
@@ -7170,7 +7170,7 @@
         <v>9</v>
       </c>
       <c r="H94" s="11">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="I94" s="11" t="s">
         <v>1</v>
@@ -7199,7 +7199,7 @@
         <v>9</v>
       </c>
       <c r="H95" s="13">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="I95" s="13" t="s">
         <v>1</v>
@@ -7228,7 +7228,7 @@
         <v>9</v>
       </c>
       <c r="H96" s="11">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="I96" s="11" t="s">
         <v>1</v>
@@ -7257,7 +7257,7 @@
         <v>9</v>
       </c>
       <c r="H97" s="13">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="I97" s="13" t="s">
         <v>1</v>
@@ -7286,7 +7286,7 @@
         <v>9</v>
       </c>
       <c r="H98" s="11">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="I98" s="11" t="s">
         <v>1</v>
@@ -7315,7 +7315,7 @@
         <v>9</v>
       </c>
       <c r="H99" s="13">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="I99" s="13" t="s">
         <v>1</v>
@@ -7344,7 +7344,7 @@
         <v>9</v>
       </c>
       <c r="H100" s="11">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I100" s="11" t="s">
         <v>1</v>
@@ -7373,7 +7373,7 @@
         <v>9</v>
       </c>
       <c r="H101" s="13">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="I101" s="13" t="s">
         <v>1</v>
@@ -7402,7 +7402,7 @@
         <v>9</v>
       </c>
       <c r="H102" s="11">
-        <v>38</v>
+        <v>83</v>
       </c>
       <c r="I102" s="11" t="s">
         <v>1</v>
@@ -7431,7 +7431,7 @@
         <v>9</v>
       </c>
       <c r="H103" s="13">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I103" s="13" t="s">
         <v>1</v>
@@ -7460,7 +7460,7 @@
         <v>9</v>
       </c>
       <c r="H104" s="11">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="I104" s="11" t="s">
         <v>1</v>
@@ -7489,7 +7489,7 @@
         <v>9</v>
       </c>
       <c r="H105" s="13">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="I105" s="13" t="s">
         <v>1</v>
@@ -7518,7 +7518,7 @@
         <v>9</v>
       </c>
       <c r="H106" s="11">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I106" s="11" t="s">
         <v>1</v>
@@ -7547,7 +7547,7 @@
         <v>9</v>
       </c>
       <c r="H107" s="13">
-        <v>13</v>
+        <v>87</v>
       </c>
       <c r="I107" s="13" t="s">
         <v>1</v>
@@ -7576,7 +7576,7 @@
         <v>9</v>
       </c>
       <c r="H108" s="11">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="I108" s="11" t="s">
         <v>1</v>
@@ -7605,7 +7605,7 @@
         <v>9</v>
       </c>
       <c r="H109" s="13">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="I109" s="13" t="s">
         <v>1</v>
@@ -7634,7 +7634,7 @@
         <v>9</v>
       </c>
       <c r="H110" s="11">
-        <v>36</v>
+        <v>86</v>
       </c>
       <c r="I110" s="11" t="s">
         <v>1</v>
@@ -7663,7 +7663,7 @@
         <v>9</v>
       </c>
       <c r="H111" s="13">
-        <v>41</v>
+        <v>84</v>
       </c>
       <c r="I111" s="13" t="s">
         <v>1</v>
@@ -7692,7 +7692,7 @@
         <v>9</v>
       </c>
       <c r="H112" s="11">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="I112" s="11" t="s">
         <v>1</v>
@@ -7721,7 +7721,7 @@
         <v>9</v>
       </c>
       <c r="H113" s="13">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="I113" s="13" t="s">
         <v>1</v>
@@ -7750,7 +7750,7 @@
         <v>9</v>
       </c>
       <c r="H114" s="11">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="I114" s="11" t="s">
         <v>1</v>
@@ -7779,7 +7779,7 @@
         <v>9</v>
       </c>
       <c r="H115" s="13">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="I115" s="13" t="s">
         <v>1</v>
@@ -7808,7 +7808,7 @@
         <v>9</v>
       </c>
       <c r="H116" s="11">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="I116" s="11" t="s">
         <v>1</v>
@@ -7837,7 +7837,7 @@
         <v>9</v>
       </c>
       <c r="H117" s="13">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="I117" s="13" t="s">
         <v>1</v>
@@ -7866,7 +7866,7 @@
         <v>9</v>
       </c>
       <c r="H118" s="11">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="I118" s="11" t="s">
         <v>1</v>
@@ -7895,7 +7895,7 @@
         <v>9</v>
       </c>
       <c r="H119" s="13">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="I119" s="13" t="s">
         <v>1</v>
@@ -7924,7 +7924,7 @@
         <v>9</v>
       </c>
       <c r="H120" s="11">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="I120" s="11" t="s">
         <v>1</v>
@@ -7953,7 +7953,7 @@
         <v>9</v>
       </c>
       <c r="H121" s="13">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="I121" s="13" t="s">
         <v>1</v>
@@ -7982,7 +7982,7 @@
         <v>9</v>
       </c>
       <c r="H122" s="11">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="I122" s="11" t="s">
         <v>1</v>
@@ -8011,7 +8011,7 @@
         <v>9</v>
       </c>
       <c r="H123" s="13">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="I123" s="13" t="s">
         <v>1</v>
@@ -8040,7 +8040,7 @@
         <v>9</v>
       </c>
       <c r="H124" s="11">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I124" s="11" t="s">
         <v>1</v>
@@ -8069,7 +8069,7 @@
         <v>9</v>
       </c>
       <c r="H125" s="13">
-        <v>23</v>
+        <v>79</v>
       </c>
       <c r="I125" s="13" t="s">
         <v>1</v>
@@ -8098,7 +8098,7 @@
         <v>9</v>
       </c>
       <c r="H126" s="11">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="I126" s="11" t="s">
         <v>1</v>
@@ -8127,7 +8127,7 @@
         <v>9</v>
       </c>
       <c r="H127" s="13">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="I127" s="13" t="s">
         <v>1</v>
@@ -8156,7 +8156,7 @@
         <v>9</v>
       </c>
       <c r="H128" s="11">
-        <v>88</v>
+        <v>35</v>
       </c>
       <c r="I128" s="11" t="s">
         <v>1</v>
@@ -8185,7 +8185,7 @@
         <v>9</v>
       </c>
       <c r="H129" s="13">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="I129" s="13" t="s">
         <v>1</v>
@@ -8214,7 +8214,7 @@
         <v>9</v>
       </c>
       <c r="H130" s="11">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="I130" s="11" t="s">
         <v>1</v>
@@ -8243,7 +8243,7 @@
         <v>9</v>
       </c>
       <c r="H131" s="13">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="I131" s="13" t="s">
         <v>1</v>
@@ -8272,7 +8272,7 @@
         <v>9</v>
       </c>
       <c r="H132" s="11">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I132" s="11" t="s">
         <v>1</v>
@@ -8301,7 +8301,7 @@
         <v>9</v>
       </c>
       <c r="H133" s="13">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I133" s="13" t="s">
         <v>1</v>
@@ -8330,7 +8330,7 @@
         <v>9</v>
       </c>
       <c r="H134" s="11">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="I134" s="11" t="s">
         <v>1</v>
@@ -8359,7 +8359,7 @@
         <v>9</v>
       </c>
       <c r="H135" s="13">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="I135" s="13" t="s">
         <v>1</v>
@@ -8388,7 +8388,7 @@
         <v>9</v>
       </c>
       <c r="H136" s="11">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="I136" s="11" t="s">
         <v>1</v>
@@ -8417,7 +8417,7 @@
         <v>9</v>
       </c>
       <c r="H137" s="13">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="I137" s="13" t="s">
         <v>1</v>
@@ -8446,7 +8446,7 @@
         <v>9</v>
       </c>
       <c r="H138" s="11">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="I138" s="11" t="s">
         <v>1</v>
@@ -8475,7 +8475,7 @@
         <v>9</v>
       </c>
       <c r="H139" s="13">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="I139" s="13" t="s">
         <v>1</v>
@@ -8504,7 +8504,7 @@
         <v>9</v>
       </c>
       <c r="H140" s="11">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="I140" s="11" t="s">
         <v>1</v>
@@ -8533,7 +8533,7 @@
         <v>9</v>
       </c>
       <c r="H141" s="13">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="I141" s="13" t="s">
         <v>1</v>
@@ -8562,7 +8562,7 @@
         <v>9</v>
       </c>
       <c r="H142" s="11">
-        <v>41</v>
+        <v>89</v>
       </c>
       <c r="I142" s="11" t="s">
         <v>1</v>
@@ -8591,7 +8591,7 @@
         <v>9</v>
       </c>
       <c r="H143" s="13">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="I143" s="13" t="s">
         <v>1</v>
@@ -8620,7 +8620,7 @@
         <v>9</v>
       </c>
       <c r="H144" s="11">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="I144" s="11" t="s">
         <v>1</v>
@@ -8649,7 +8649,7 @@
         <v>9</v>
       </c>
       <c r="H145" s="13">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="I145" s="13" t="s">
         <v>1</v>
@@ -8678,7 +8678,7 @@
         <v>9</v>
       </c>
       <c r="H146" s="11">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="I146" s="11" t="s">
         <v>1</v>
@@ -8707,7 +8707,7 @@
         <v>9</v>
       </c>
       <c r="H147" s="13">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="I147" s="13" t="s">
         <v>1</v>
@@ -8736,7 +8736,7 @@
         <v>9</v>
       </c>
       <c r="H148" s="11">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="I148" s="11" t="s">
         <v>1</v>
@@ -8765,7 +8765,7 @@
         <v>9</v>
       </c>
       <c r="H149" s="13">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="I149" s="13" t="s">
         <v>1</v>
@@ -8794,7 +8794,7 @@
         <v>9</v>
       </c>
       <c r="H150" s="11">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="I150" s="11" t="s">
         <v>1</v>
@@ -8823,7 +8823,7 @@
         <v>9</v>
       </c>
       <c r="H151" s="13">
-        <v>35</v>
+        <v>63</v>
       </c>
       <c r="I151" s="13" t="s">
         <v>1</v>
@@ -8852,7 +8852,7 @@
         <v>9</v>
       </c>
       <c r="H152" s="11">
-        <v>48</v>
+        <v>85</v>
       </c>
       <c r="I152" s="11" t="s">
         <v>1</v>
@@ -8881,7 +8881,7 @@
         <v>9</v>
       </c>
       <c r="H153" s="13">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="I153" s="13" t="s">
         <v>1</v>
@@ -8910,7 +8910,7 @@
         <v>9</v>
       </c>
       <c r="H154" s="11">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="I154" s="11" t="s">
         <v>1</v>
@@ -8939,7 +8939,7 @@
         <v>9</v>
       </c>
       <c r="H155" s="13">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I155" s="13" t="s">
         <v>1</v>
@@ -8968,7 +8968,7 @@
         <v>9</v>
       </c>
       <c r="H156" s="11">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="I156" s="11" t="s">
         <v>1</v>
@@ -8997,7 +8997,7 @@
         <v>9</v>
       </c>
       <c r="H157" s="13">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="I157" s="13" t="s">
         <v>1</v>
@@ -9026,7 +9026,7 @@
         <v>9</v>
       </c>
       <c r="H158" s="11">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="I158" s="11" t="s">
         <v>1</v>
@@ -9055,7 +9055,7 @@
         <v>9</v>
       </c>
       <c r="H159" s="13">
-        <v>73</v>
+        <v>36</v>
       </c>
       <c r="I159" s="13" t="s">
         <v>1</v>
@@ -9084,7 +9084,7 @@
         <v>9</v>
       </c>
       <c r="H160" s="11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="I160" s="11" t="s">
         <v>1</v>
@@ -9113,7 +9113,7 @@
         <v>9</v>
       </c>
       <c r="H161" s="13">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="I161" s="13" t="s">
         <v>1</v>
@@ -9142,7 +9142,7 @@
         <v>9</v>
       </c>
       <c r="H162" s="11">
-        <v>43</v>
+        <v>75</v>
       </c>
       <c r="I162" s="11" t="s">
         <v>1</v>
@@ -9171,7 +9171,7 @@
         <v>9</v>
       </c>
       <c r="H163" s="13">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I163" s="13" t="s">
         <v>1</v>
@@ -9200,7 +9200,7 @@
         <v>9</v>
       </c>
       <c r="H164" s="11">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="I164" s="11" t="s">
         <v>1</v>
@@ -9229,7 +9229,7 @@
         <v>9</v>
       </c>
       <c r="H165" s="13">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="I165" s="13" t="s">
         <v>1</v>
@@ -9258,7 +9258,7 @@
         <v>9</v>
       </c>
       <c r="H166" s="11">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="I166" s="11" t="s">
         <v>1</v>
@@ -9287,7 +9287,7 @@
         <v>9</v>
       </c>
       <c r="H167" s="13">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="I167" s="13" t="s">
         <v>1</v>
@@ -9316,7 +9316,7 @@
         <v>9</v>
       </c>
       <c r="H168" s="11">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="I168" s="11" t="s">
         <v>1</v>
@@ -9345,7 +9345,7 @@
         <v>9</v>
       </c>
       <c r="H169" s="13">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="I169" s="13" t="s">
         <v>1</v>
@@ -9374,7 +9374,7 @@
         <v>9</v>
       </c>
       <c r="H170" s="11">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="I170" s="11" t="s">
         <v>1</v>
@@ -9403,7 +9403,7 @@
         <v>9</v>
       </c>
       <c r="H171" s="13">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="I171" s="13" t="s">
         <v>1</v>
@@ -9432,7 +9432,7 @@
         <v>9</v>
       </c>
       <c r="H172" s="11">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="I172" s="11" t="s">
         <v>1</v>
@@ -9461,7 +9461,7 @@
         <v>9</v>
       </c>
       <c r="H173" s="13">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="I173" s="13" t="s">
         <v>1</v>
@@ -9490,7 +9490,7 @@
         <v>9</v>
       </c>
       <c r="H174" s="11">
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="I174" s="11" t="s">
         <v>1</v>
@@ -9519,7 +9519,7 @@
         <v>9</v>
       </c>
       <c r="H175" s="13">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="I175" s="13" t="s">
         <v>1</v>
@@ -9548,7 +9548,7 @@
         <v>9</v>
       </c>
       <c r="H176" s="11">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="I176" s="11" t="s">
         <v>1</v>
@@ -9577,7 +9577,7 @@
         <v>9</v>
       </c>
       <c r="H177" s="13">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="I177" s="13" t="s">
         <v>1</v>
@@ -9606,7 +9606,7 @@
         <v>9</v>
       </c>
       <c r="H178" s="11">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="I178" s="11" t="s">
         <v>1</v>
@@ -9635,7 +9635,7 @@
         <v>9</v>
       </c>
       <c r="H179" s="13">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="I179" s="13" t="s">
         <v>1</v>
@@ -9664,7 +9664,7 @@
         <v>9</v>
       </c>
       <c r="H180" s="11">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="I180" s="11" t="s">
         <v>1</v>
@@ -9693,7 +9693,7 @@
         <v>9</v>
       </c>
       <c r="H181" s="13">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="I181" s="13" t="s">
         <v>1</v>
@@ -9722,7 +9722,7 @@
         <v>9</v>
       </c>
       <c r="H182" s="11">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I182" s="11" t="s">
         <v>1</v>
@@ -9751,7 +9751,7 @@
         <v>9</v>
       </c>
       <c r="H183" s="13">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="I183" s="13" t="s">
         <v>1</v>
@@ -9780,7 +9780,7 @@
         <v>9</v>
       </c>
       <c r="H184" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="I184" s="11" t="s">
         <v>1</v>
@@ -9809,7 +9809,7 @@
         <v>9</v>
       </c>
       <c r="H185" s="13">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="I185" s="13" t="s">
         <v>1</v>
@@ -9838,7 +9838,7 @@
         <v>9</v>
       </c>
       <c r="H186" s="11">
-        <v>41</v>
+        <v>77</v>
       </c>
       <c r="I186" s="11" t="s">
         <v>1</v>
@@ -9867,7 +9867,7 @@
         <v>9</v>
       </c>
       <c r="H187" s="13">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="I187" s="13" t="s">
         <v>1</v>
@@ -9896,7 +9896,7 @@
         <v>9</v>
       </c>
       <c r="H188" s="11">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="I188" s="11" t="s">
         <v>1</v>
@@ -9925,7 +9925,7 @@
         <v>9</v>
       </c>
       <c r="H189" s="13">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="I189" s="13" t="s">
         <v>1</v>
@@ -9954,7 +9954,7 @@
         <v>9</v>
       </c>
       <c r="H190" s="11">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="I190" s="11" t="s">
         <v>1</v>
@@ -9983,7 +9983,7 @@
         <v>9</v>
       </c>
       <c r="H191" s="13">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="I191" s="13" t="s">
         <v>1</v>
@@ -10012,7 +10012,7 @@
         <v>9</v>
       </c>
       <c r="H192" s="11">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="I192" s="11" t="s">
         <v>1</v>
@@ -10041,7 +10041,7 @@
         <v>9</v>
       </c>
       <c r="H193" s="13">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="I193" s="13" t="s">
         <v>1</v>
@@ -10070,7 +10070,7 @@
         <v>9</v>
       </c>
       <c r="H194" s="11">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="I194" s="11" t="s">
         <v>1</v>
@@ -10099,7 +10099,7 @@
         <v>9</v>
       </c>
       <c r="H195" s="13">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="I195" s="13" t="s">
         <v>1</v>
@@ -10128,7 +10128,7 @@
         <v>9</v>
       </c>
       <c r="H196" s="11">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="I196" s="11" t="s">
         <v>1</v>
@@ -10157,7 +10157,7 @@
         <v>9</v>
       </c>
       <c r="H197" s="13">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="I197" s="13" t="s">
         <v>1</v>
@@ -10186,7 +10186,7 @@
         <v>9</v>
       </c>
       <c r="H198" s="11">
-        <v>85</v>
+        <v>51</v>
       </c>
       <c r="I198" s="11" t="s">
         <v>1</v>
@@ -10215,7 +10215,7 @@
         <v>9</v>
       </c>
       <c r="H199" s="13">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="I199" s="13" t="s">
         <v>1</v>
@@ -10244,7 +10244,7 @@
         <v>9</v>
       </c>
       <c r="H200" s="11">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="I200" s="11" t="s">
         <v>1</v>
@@ -10302,7 +10302,7 @@
         <v>9</v>
       </c>
       <c r="H202" s="11">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="I202" s="11" t="s">
         <v>1</v>
@@ -10331,7 +10331,7 @@
         <v>9</v>
       </c>
       <c r="H203" s="13">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I203" s="13" t="s">
         <v>1</v>
@@ -10360,7 +10360,7 @@
         <v>9</v>
       </c>
       <c r="H204" s="11">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="I204" s="11" t="s">
         <v>1</v>
@@ -10389,7 +10389,7 @@
         <v>9</v>
       </c>
       <c r="H205" s="13">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="I205" s="13" t="s">
         <v>1</v>
@@ -10418,7 +10418,7 @@
         <v>9</v>
       </c>
       <c r="H206" s="11">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="I206" s="11" t="s">
         <v>1</v>
@@ -10447,7 +10447,7 @@
         <v>9</v>
       </c>
       <c r="H207" s="13">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="I207" s="13" t="s">
         <v>1</v>
@@ -10476,7 +10476,7 @@
         <v>9</v>
       </c>
       <c r="H208" s="11">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="I208" s="11" t="s">
         <v>1</v>
@@ -10505,7 +10505,7 @@
         <v>9</v>
       </c>
       <c r="H209" s="13">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="I209" s="13" t="s">
         <v>1</v>
@@ -10534,7 +10534,7 @@
         <v>9</v>
       </c>
       <c r="H210" s="11">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="I210" s="11" t="s">
         <v>1</v>
@@ -10563,7 +10563,7 @@
         <v>9</v>
       </c>
       <c r="H211" s="13">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="I211" s="13" t="s">
         <v>1</v>
@@ -10592,7 +10592,7 @@
         <v>9</v>
       </c>
       <c r="H212" s="11">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="I212" s="11" t="s">
         <v>1</v>
@@ -10621,7 +10621,7 @@
         <v>9</v>
       </c>
       <c r="H213" s="13">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="I213" s="13" t="s">
         <v>1</v>
@@ -10650,7 +10650,7 @@
         <v>9</v>
       </c>
       <c r="H214" s="11">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="I214" s="11" t="s">
         <v>1</v>
@@ -10679,7 +10679,7 @@
         <v>9</v>
       </c>
       <c r="H215" s="13">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="I215" s="13" t="s">
         <v>1</v>
@@ -10708,7 +10708,7 @@
         <v>9</v>
       </c>
       <c r="H216" s="11">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="I216" s="11" t="s">
         <v>1</v>
@@ -10737,7 +10737,7 @@
         <v>9</v>
       </c>
       <c r="H217" s="13">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="I217" s="13" t="s">
         <v>1</v>
@@ -10766,7 +10766,7 @@
         <v>9</v>
       </c>
       <c r="H218" s="11">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="I218" s="11" t="s">
         <v>1</v>
@@ -10795,7 +10795,7 @@
         <v>9</v>
       </c>
       <c r="H219" s="13">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="I219" s="13" t="s">
         <v>1</v>
@@ -10824,7 +10824,7 @@
         <v>9</v>
       </c>
       <c r="H220" s="11">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="I220" s="11" t="s">
         <v>1</v>
@@ -10853,7 +10853,7 @@
         <v>9</v>
       </c>
       <c r="H221" s="13">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="I221" s="13" t="s">
         <v>1</v>
@@ -10882,7 +10882,7 @@
         <v>9</v>
       </c>
       <c r="H222" s="11">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="I222" s="11" t="s">
         <v>1</v>
@@ -10911,7 +10911,7 @@
         <v>9</v>
       </c>
       <c r="H223" s="13">
-        <v>43</v>
+        <v>85</v>
       </c>
       <c r="I223" s="13" t="s">
         <v>1</v>
@@ -10940,7 +10940,7 @@
         <v>9</v>
       </c>
       <c r="H224" s="11">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="I224" s="11" t="s">
         <v>1</v>
@@ -10969,7 +10969,7 @@
         <v>9</v>
       </c>
       <c r="H225" s="13">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="I225" s="13" t="s">
         <v>1</v>
@@ -10998,7 +10998,7 @@
         <v>9</v>
       </c>
       <c r="H226" s="11">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="I226" s="11" t="s">
         <v>1</v>
@@ -11027,7 +11027,7 @@
         <v>9</v>
       </c>
       <c r="H227" s="13">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="I227" s="13" t="s">
         <v>1</v>
@@ -11056,7 +11056,7 @@
         <v>9</v>
       </c>
       <c r="H228" s="11">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="I228" s="11" t="s">
         <v>1</v>
@@ -11085,7 +11085,7 @@
         <v>9</v>
       </c>
       <c r="H229" s="13">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="I229" s="13" t="s">
         <v>1</v>
@@ -11114,7 +11114,7 @@
         <v>9</v>
       </c>
       <c r="H230" s="11">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="I230" s="11" t="s">
         <v>1</v>
@@ -11143,7 +11143,7 @@
         <v>9</v>
       </c>
       <c r="H231" s="13">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="I231" s="13" t="s">
         <v>1</v>
@@ -11172,7 +11172,7 @@
         <v>9</v>
       </c>
       <c r="H232" s="11">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="I232" s="11" t="s">
         <v>1</v>
@@ -11201,7 +11201,7 @@
         <v>9</v>
       </c>
       <c r="H233" s="13">
-        <v>88</v>
+        <v>29</v>
       </c>
       <c r="I233" s="13" t="s">
         <v>1</v>
@@ -11230,7 +11230,7 @@
         <v>9</v>
       </c>
       <c r="H234" s="11">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="I234" s="11" t="s">
         <v>1</v>
@@ -11259,7 +11259,7 @@
         <v>9</v>
       </c>
       <c r="H235" s="13">
-        <v>81</v>
+        <v>54</v>
       </c>
       <c r="I235" s="13" t="s">
         <v>1</v>
@@ -11288,7 +11288,7 @@
         <v>9</v>
       </c>
       <c r="H236" s="11">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="I236" s="11" t="s">
         <v>1</v>
@@ -11317,7 +11317,7 @@
         <v>9</v>
       </c>
       <c r="H237" s="13">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="I237" s="13" t="s">
         <v>1</v>
@@ -11346,7 +11346,7 @@
         <v>9</v>
       </c>
       <c r="H238" s="11">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="I238" s="11" t="s">
         <v>1</v>
@@ -11375,7 +11375,7 @@
         <v>9</v>
       </c>
       <c r="H239" s="13">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="I239" s="13" t="s">
         <v>1</v>
@@ -11404,7 +11404,7 @@
         <v>9</v>
       </c>
       <c r="H240" s="11">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="I240" s="11" t="s">
         <v>1</v>
@@ -11433,7 +11433,7 @@
         <v>9</v>
       </c>
       <c r="H241" s="13">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="I241" s="13" t="s">
         <v>1</v>
@@ -11462,7 +11462,7 @@
         <v>9</v>
       </c>
       <c r="H242" s="11">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="I242" s="11" t="s">
         <v>1</v>
@@ -11491,7 +11491,7 @@
         <v>9</v>
       </c>
       <c r="H243" s="13">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I243" s="13" t="s">
         <v>1</v>
@@ -11520,7 +11520,7 @@
         <v>9</v>
       </c>
       <c r="H244" s="11">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="I244" s="11" t="s">
         <v>1</v>
@@ -11549,7 +11549,7 @@
         <v>9</v>
       </c>
       <c r="H245" s="13">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="I245" s="13" t="s">
         <v>1</v>
@@ -11578,7 +11578,7 @@
         <v>9</v>
       </c>
       <c r="H246" s="11">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="I246" s="11" t="s">
         <v>1</v>
@@ -11607,7 +11607,7 @@
         <v>9</v>
       </c>
       <c r="H247" s="13">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="I247" s="13" t="s">
         <v>1</v>
@@ -11636,7 +11636,7 @@
         <v>9</v>
       </c>
       <c r="H248" s="11">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="I248" s="11" t="s">
         <v>1</v>
@@ -11665,7 +11665,7 @@
         <v>9</v>
       </c>
       <c r="H249" s="13">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="I249" s="13" t="s">
         <v>1</v>
@@ -11694,7 +11694,7 @@
         <v>9</v>
       </c>
       <c r="H250" s="11">
-        <v>10</v>
+        <v>53</v>
       </c>
       <c r="I250" s="11" t="s">
         <v>1</v>
@@ -11723,7 +11723,7 @@
         <v>9</v>
       </c>
       <c r="H251" s="13">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I251" s="13" t="s">
         <v>1</v>
@@ -11752,7 +11752,7 @@
         <v>9</v>
       </c>
       <c r="H252" s="11">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="I252" s="11" t="s">
         <v>1</v>
@@ -11772,7 +11772,7 @@
         <v>960</v>
       </c>
       <c r="E253" s="13" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="F253" s="13" t="s">
         <v>957</v>
@@ -11781,7 +11781,7 @@
         <v>9</v>
       </c>
       <c r="H253" s="13">
-        <v>54</v>
+        <v>82</v>
       </c>
       <c r="I253" s="13" t="s">
         <v>1</v>
@@ -11789,19 +11789,19 @@
     </row>
     <row r="254" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A254" s="11" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="B254" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C254" s="11" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="D254" s="11" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="E254" s="11" t="s">
-        <v>964</v>
+        <v>956</v>
       </c>
       <c r="F254" s="11" t="s">
         <v>957</v>
@@ -11810,7 +11810,7 @@
         <v>9</v>
       </c>
       <c r="H254" s="11">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="I254" s="11" t="s">
         <v>1</v>
@@ -11839,7 +11839,7 @@
         <v>9</v>
       </c>
       <c r="H255" s="13">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="I255" s="13" t="s">
         <v>1</v>
@@ -11859,7 +11859,7 @@
         <v>971</v>
       </c>
       <c r="E256" s="11" t="s">
-        <v>964</v>
+        <v>956</v>
       </c>
       <c r="F256" s="11" t="s">
         <v>957</v>
@@ -11868,7 +11868,7 @@
         <v>9</v>
       </c>
       <c r="H256" s="11">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="I256" s="11" t="s">
         <v>1</v>
@@ -11888,7 +11888,7 @@
         <v>974</v>
       </c>
       <c r="E257" s="13" t="s">
-        <v>956</v>
+        <v>968</v>
       </c>
       <c r="F257" s="13" t="s">
         <v>957</v>
@@ -11897,7 +11897,7 @@
         <v>9</v>
       </c>
       <c r="H257" s="13">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="I257" s="13" t="s">
         <v>1</v>
@@ -11926,7 +11926,7 @@
         <v>9</v>
       </c>
       <c r="H258" s="11">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="I258" s="11" t="s">
         <v>1</v>
@@ -11943,10 +11943,10 @@
         <v>979</v>
       </c>
       <c r="D259" s="13" t="s">
-        <v>980</v>
+        <v>967</v>
       </c>
       <c r="E259" s="13" t="s">
-        <v>956</v>
+        <v>968</v>
       </c>
       <c r="F259" s="13" t="s">
         <v>957</v>
@@ -11955,7 +11955,7 @@
         <v>9</v>
       </c>
       <c r="H259" s="13">
-        <v>87</v>
+        <v>54</v>
       </c>
       <c r="I259" s="13" t="s">
         <v>1</v>
@@ -11963,19 +11963,19 @@
     </row>
     <row r="260" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A260" s="11" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B260" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C260" s="11" t="s">
+        <v>981</v>
+      </c>
+      <c r="D260" s="11" t="s">
         <v>982</v>
       </c>
-      <c r="D260" s="11" t="s">
-        <v>960</v>
-      </c>
       <c r="E260" s="11" t="s">
-        <v>956</v>
+        <v>968</v>
       </c>
       <c r="F260" s="11" t="s">
         <v>957</v>
@@ -11984,7 +11984,7 @@
         <v>9</v>
       </c>
       <c r="H260" s="11">
-        <v>13</v>
+        <v>68</v>
       </c>
       <c r="I260" s="11" t="s">
         <v>1</v>
@@ -12001,10 +12001,10 @@
         <v>984</v>
       </c>
       <c r="D261" s="13" t="s">
-        <v>960</v>
+        <v>985</v>
       </c>
       <c r="E261" s="13" t="s">
-        <v>956</v>
+        <v>968</v>
       </c>
       <c r="F261" s="13" t="s">
         <v>957</v>
@@ -12013,7 +12013,7 @@
         <v>9</v>
       </c>
       <c r="H261" s="13">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="I261" s="13" t="s">
         <v>1</v>
@@ -12021,19 +12021,19 @@
     </row>
     <row r="262" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A262" s="11" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="B262" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C262" s="11" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="D262" s="11" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="E262" s="11" t="s">
-        <v>964</v>
+        <v>968</v>
       </c>
       <c r="F262" s="11" t="s">
         <v>957</v>
@@ -12042,7 +12042,7 @@
         <v>9</v>
       </c>
       <c r="H262" s="11">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="I262" s="11" t="s">
         <v>1</v>
@@ -12050,19 +12050,19 @@
     </row>
     <row r="263" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A263" s="13" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="B263" s="13" t="s">
         <v>24</v>
       </c>
       <c r="C263" s="13" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="D263" s="13" t="s">
-        <v>990</v>
+        <v>971</v>
       </c>
       <c r="E263" s="13" t="s">
-        <v>964</v>
+        <v>956</v>
       </c>
       <c r="F263" s="13" t="s">
         <v>957</v>
@@ -12071,7 +12071,7 @@
         <v>9</v>
       </c>
       <c r="H263" s="13">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="I263" s="13" t="s">
         <v>1</v>
@@ -12100,7 +12100,7 @@
         <v>9</v>
       </c>
       <c r="H264" s="11">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="I264" s="11" t="s">
         <v>1</v>
@@ -12120,7 +12120,7 @@
         <v>996</v>
       </c>
       <c r="E265" s="13" t="s">
-        <v>964</v>
+        <v>956</v>
       </c>
       <c r="F265" s="13" t="s">
         <v>957</v>
@@ -12129,7 +12129,7 @@
         <v>9</v>
       </c>
       <c r="H265" s="13">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="I265" s="13" t="s">
         <v>1</v>
@@ -12149,7 +12149,7 @@
         <v>999</v>
       </c>
       <c r="E266" s="11" t="s">
-        <v>956</v>
+        <v>968</v>
       </c>
       <c r="F266" s="11" t="s">
         <v>957</v>
@@ -12158,7 +12158,7 @@
         <v>9</v>
       </c>
       <c r="H266" s="11">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="I266" s="11" t="s">
         <v>1</v>
@@ -12178,7 +12178,7 @@
         <v>1002</v>
       </c>
       <c r="E267" s="13" t="s">
-        <v>956</v>
+        <v>968</v>
       </c>
       <c r="F267" s="13" t="s">
         <v>957</v>
@@ -12187,7 +12187,7 @@
         <v>9</v>
       </c>
       <c r="H267" s="13">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="I267" s="13" t="s">
         <v>1</v>
@@ -12216,7 +12216,7 @@
         <v>9</v>
       </c>
       <c r="H268" s="11">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I268" s="11" t="s">
         <v>1</v>
@@ -12245,7 +12245,7 @@
         <v>9</v>
       </c>
       <c r="H269" s="13">
-        <v>80</v>
+        <v>36</v>
       </c>
       <c r="I269" s="13" t="s">
         <v>1</v>
@@ -12274,7 +12274,7 @@
         <v>9</v>
       </c>
       <c r="H270" s="11">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="I270" s="11" t="s">
         <v>1</v>
@@ -12303,7 +12303,7 @@
         <v>9</v>
       </c>
       <c r="H271" s="13">
-        <v>82</v>
+        <v>43</v>
       </c>
       <c r="I271" s="13" t="s">
         <v>1</v>
@@ -12332,7 +12332,7 @@
         <v>9</v>
       </c>
       <c r="H272" s="11">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="I272" s="11" t="s">
         <v>1</v>
@@ -12361,7 +12361,7 @@
         <v>9</v>
       </c>
       <c r="H273" s="13">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="I273" s="13" t="s">
         <v>1</v>
@@ -12390,7 +12390,7 @@
         <v>9</v>
       </c>
       <c r="H274" s="11">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="I274" s="11" t="s">
         <v>1</v>
@@ -12419,7 +12419,7 @@
         <v>9</v>
       </c>
       <c r="H275" s="13">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="I275" s="13" t="s">
         <v>1</v>
@@ -12448,7 +12448,7 @@
         <v>9</v>
       </c>
       <c r="H276" s="11">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="I276" s="11" t="s">
         <v>1</v>
@@ -12477,7 +12477,7 @@
         <v>9</v>
       </c>
       <c r="H277" s="13">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="I277" s="13" t="s">
         <v>1</v>
@@ -12506,7 +12506,7 @@
         <v>9</v>
       </c>
       <c r="H278" s="11">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="I278" s="11" t="s">
         <v>1</v>
@@ -12535,7 +12535,7 @@
         <v>9</v>
       </c>
       <c r="H279" s="13">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="I279" s="13" t="s">
         <v>1</v>
@@ -12564,7 +12564,7 @@
         <v>9</v>
       </c>
       <c r="H280" s="11">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="I280" s="11" t="s">
         <v>1</v>
@@ -12593,7 +12593,7 @@
         <v>9</v>
       </c>
       <c r="H281" s="13">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="I281" s="13" t="s">
         <v>1</v>
@@ -12622,7 +12622,7 @@
         <v>9</v>
       </c>
       <c r="H282" s="11">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="I282" s="11" t="s">
         <v>1</v>
@@ -12651,7 +12651,7 @@
         <v>9</v>
       </c>
       <c r="H283" s="13">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="I283" s="13" t="s">
         <v>1</v>
@@ -12680,7 +12680,7 @@
         <v>9</v>
       </c>
       <c r="H284" s="11">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="I284" s="11" t="s">
         <v>1</v>
@@ -12709,7 +12709,7 @@
         <v>9</v>
       </c>
       <c r="H285" s="13">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I285" s="13" t="s">
         <v>1</v>
@@ -12738,7 +12738,7 @@
         <v>9</v>
       </c>
       <c r="H286" s="11">
-        <v>71</v>
+        <v>22</v>
       </c>
       <c r="I286" s="11" t="s">
         <v>1</v>
@@ -12767,7 +12767,7 @@
         <v>9</v>
       </c>
       <c r="H287" s="13">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="I287" s="13" t="s">
         <v>1</v>
@@ -12796,7 +12796,7 @@
         <v>9</v>
       </c>
       <c r="H288" s="11">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="I288" s="11" t="s">
         <v>1</v>
@@ -12825,7 +12825,7 @@
         <v>9</v>
       </c>
       <c r="H289" s="13">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="I289" s="13" t="s">
         <v>1</v>
@@ -12854,7 +12854,7 @@
         <v>9</v>
       </c>
       <c r="H290" s="11">
-        <v>24</v>
+        <v>68</v>
       </c>
       <c r="I290" s="11" t="s">
         <v>1</v>
@@ -12883,7 +12883,7 @@
         <v>9</v>
       </c>
       <c r="H291" s="13">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I291" s="13" t="s">
         <v>1</v>
@@ -12912,7 +12912,7 @@
         <v>9</v>
       </c>
       <c r="H292" s="11">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I292" s="11" t="s">
         <v>1</v>
@@ -12941,7 +12941,7 @@
         <v>9</v>
       </c>
       <c r="H293" s="13">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="I293" s="13" t="s">
         <v>1</v>
@@ -12970,7 +12970,7 @@
         <v>9</v>
       </c>
       <c r="H294" s="11">
-        <v>69</v>
+        <v>38</v>
       </c>
       <c r="I294" s="11" t="s">
         <v>1</v>
@@ -12999,7 +12999,7 @@
         <v>9</v>
       </c>
       <c r="H295" s="13">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="I295" s="13" t="s">
         <v>1</v>
@@ -13028,7 +13028,7 @@
         <v>9</v>
       </c>
       <c r="H296" s="11">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="I296" s="11" t="s">
         <v>1</v>
@@ -13057,7 +13057,7 @@
         <v>9</v>
       </c>
       <c r="H297" s="13">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="I297" s="13" t="s">
         <v>1</v>
@@ -13086,7 +13086,7 @@
         <v>9</v>
       </c>
       <c r="H298" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I298" s="11" t="s">
         <v>1</v>
@@ -13115,7 +13115,7 @@
         <v>9</v>
       </c>
       <c r="H299" s="13">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="I299" s="13" t="s">
         <v>1</v>
@@ -13144,7 +13144,7 @@
         <v>9</v>
       </c>
       <c r="H300" s="11">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="I300" s="11" t="s">
         <v>1</v>
@@ -13173,7 +13173,7 @@
         <v>9</v>
       </c>
       <c r="H301" s="13">
-        <v>11</v>
+        <v>77</v>
       </c>
       <c r="I301" s="13" t="s">
         <v>1</v>

</xml_diff>